<commit_message>
Update published master datasets (2026-02-24)
</commit_message>
<xml_diff>
--- a/archive/InnovateUK_Funding_Opportunities_Latest_2026-02-24.xlsx
+++ b/archive/InnovateUK_Funding_Opportunities_Latest_2026-02-24.xlsx
@@ -1257,7 +1257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1335,26 +1335,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Innovate UK Business Connect</t>
+          <t>Innovate Funding Service</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Semiconductors and components for smart electronic platforms</t>
+          <t>Robotics Adoption Hubs</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/semiconductors-and-components-for-smart-electronic-platforms/</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2408/overview/ad7d7d36-af60-48be-91b0-f3208cf7c1d4</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-02-23 10:38</t>
+          <t>2026-02-24 10:43</t>
         </is>
       </c>
       <c r="E2" s="1" t="n">
-        <v>46076.44305555556</v>
+        <v>46077.44652777778</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -1363,25 +1363,19 @@
       <c r="H2" t="b">
         <v>0</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>20/02/2026</t>
-        </is>
-      </c>
-      <c r="J2" s="1" t="n">
-        <v>46073</v>
-      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
-          <t>01/04/2026                              11:00</t>
+          <t>Wednesday 15 April 2026 11:00am</t>
         </is>
       </c>
       <c r="L2" s="1" t="n">
-        <v>46113.45833333334</v>
+        <v>46127.45833333334</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>£18.5 million</t>
+          <t>£7.5 million</t>
         </is>
       </c>
       <c r="N2" s="1" t="n">
@@ -1391,26 +1385,26 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Innovate UK Business Connect</t>
+          <t>Innovate Funding Service</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>iX Challenge - Dry ice alternatives that maintain LUSH spa's sensory and theatrical magic</t>
+          <t>Robotics Adoption Central Convening Body</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-dry-ice-alternatives-maintaining-lush-spas-sensory-and-theatrical-magic/</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2409/overview/c7e5dd6a-9f34-4614-b548-214b76190c14</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-02-23 10:38</t>
+          <t>2026-02-24 10:43</t>
         </is>
       </c>
       <c r="E3" s="1" t="n">
-        <v>46076.44305555556</v>
+        <v>46077.44652777778</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -1419,25 +1413,19 @@
       <c r="H3" t="b">
         <v>0</v>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>23/02/2026</t>
-        </is>
-      </c>
-      <c r="J3" s="1" t="n">
-        <v>46076</v>
-      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
-          <t>17/04/2026                              23:59</t>
+          <t>Wednesday 15 April 2026 11:00am</t>
         </is>
       </c>
       <c r="L3" s="1" t="n">
-        <v>46129.99930555555</v>
+        <v>46127.45833333334</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>£99</t>
+          <t>£2.0 million</t>
         </is>
       </c>
       <c r="N3" s="1" t="n">
@@ -1452,21 +1440,21 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: industrial human relevant drug models</t>
+          <t>iX Challenge - Enabling regional carbon dioxide utilisation in Southwest Wales through geospatial intelligence</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/contracts-for-innovation-industrial-human-relevant-drug-models/</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-enabling-regional-carbon-dioxide-utilisation-southwest-wales/</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-02-21 10:13</t>
+          <t>2026-02-24 10:36</t>
         </is>
       </c>
       <c r="E4" s="1" t="n">
-        <v>46074.42569444444</v>
+        <v>46077.44166666667</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -1477,23 +1465,23 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>02/03/2026</t>
+          <t>24/02/2026</t>
         </is>
       </c>
       <c r="J4" s="1" t="n">
-        <v>46083</v>
+        <v>46077</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>15/04/2026                              11:00</t>
+          <t>23/04/2026                              23:59</t>
         </is>
       </c>
       <c r="L4" s="1" t="n">
-        <v>46127.45833333334</v>
+        <v>46135.99930555555</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>£2.0 million</t>
+          <t>£25,000</t>
         </is>
       </c>
       <c r="N4" s="1" t="n">
@@ -1503,7 +1491,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1513,16 +1501,16 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2403/overview/4b54c133-c9b2-4572-9cca-2a7a4f69e5b8</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/semiconductors-and-components-for-smart-electronic-platforms/</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-02-20 10:32</t>
+          <t>2026-02-23 10:38</t>
         </is>
       </c>
       <c r="E5" s="1" t="n">
-        <v>46073.43888888889</v>
+        <v>46076.44305555556</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
@@ -1531,11 +1519,17 @@
       <c r="H5" t="b">
         <v>0</v>
       </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>20/02/2026</t>
+        </is>
+      </c>
+      <c r="J5" s="1" t="n">
+        <v>46073</v>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Wednesday 1 April 2026 11:00am</t>
+          <t>01/04/2026                              11:00</t>
         </is>
       </c>
       <c r="L5" s="1" t="n">
@@ -1543,7 +1537,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>£2.0 million</t>
+          <t>£18.5 million</t>
         </is>
       </c>
       <c r="N5" s="1" t="n">
@@ -1558,21 +1552,21 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AI Management Practitioner Training</t>
+          <t>iX Challenge - Dry ice alternatives that maintain LUSH spa's sensory and theatrical magic</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/ai-management-practitioner-training/</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-dry-ice-alternatives-maintaining-lush-spas-sensory-and-theatrical-magic/</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-02-20 10:25</t>
+          <t>2026-02-23 10:38</t>
         </is>
       </c>
       <c r="E6" s="1" t="n">
-        <v>46073.43402777778</v>
+        <v>46076.44305555556</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
@@ -1581,11 +1575,27 @@
       <c r="H6" t="b">
         <v>0</v>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>23/02/2026</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="n">
+        <v>46076</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>17/04/2026                              23:59</t>
+        </is>
+      </c>
+      <c r="L6" s="1" t="n">
+        <v>46129.99930555555</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>£99</t>
+        </is>
+      </c>
       <c r="N6" s="1" t="n">
         <v>46071</v>
       </c>
@@ -1598,21 +1608,21 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Southwest Wales Net Zero Industry Launchpad Round 2 - Call for challenge holders</t>
+          <t>Contracts for Innovation: industrial human relevant drug models</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://iuk-business-connect.org.uk/opportunities/southwest-wales-net-zero-industry-launchpad-round-2-call-for-challenge-holders/</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/contracts-for-innovation-industrial-human-relevant-drug-models/</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-02-18 10:32</t>
+          <t>2026-02-21 10:13</t>
         </is>
       </c>
       <c r="E7" s="1" t="n">
-        <v>46071.43888888889</v>
+        <v>46074.42569444444</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
@@ -1623,26 +1633,172 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
+          <t>02/03/2026</t>
+        </is>
+      </c>
+      <c r="J7" s="1" t="n">
+        <v>46083</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>15/04/2026                              11:00</t>
+        </is>
+      </c>
+      <c r="L7" s="1" t="n">
+        <v>46127.45833333334</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>£2.0 million</t>
+        </is>
+      </c>
+      <c r="N7" s="1" t="n">
+        <v>46071</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Semiconductors and components for smart electronic platforms</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2403/overview/4b54c133-c9b2-4572-9cca-2a7a4f69e5b8</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-02-20 10:32</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>46073.43888888889</v>
+      </c>
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Wednesday 1 April 2026 11:00am</t>
+        </is>
+      </c>
+      <c r="L8" s="1" t="n">
+        <v>46113.45833333334</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>£2.0 million</t>
+        </is>
+      </c>
+      <c r="N8" s="1" t="n">
+        <v>46071</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Innovate UK Business Connect</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>AI Management Practitioner Training</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://iuk-business-connect.org.uk/opportunities/ai-management-practitioner-training/</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-02-20 10:25</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>46073.43402777778</v>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="b">
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" s="1" t="n">
+        <v>46071</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Innovate UK Business Connect</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Southwest Wales Net Zero Industry Launchpad Round 2 - Call for challenge holders</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://iuk-business-connect.org.uk/opportunities/southwest-wales-net-zero-industry-launchpad-round-2-call-for-challenge-holders/</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-02-18 10:32</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>46071.43888888889</v>
+      </c>
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="b">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
           <t>18/02/2026</t>
         </is>
       </c>
-      <c r="J7" s="1" t="n">
+      <c r="J10" s="1" t="n">
         <v>46071</v>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>13/03/2026                              00:00</t>
         </is>
       </c>
-      <c r="L7" s="1" t="n">
+      <c r="L10" s="1" t="n">
         <v>46094</v>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>£25,000</t>
         </is>
       </c>
-      <c r="N7" s="1" t="n">
+      <c r="N10" s="1" t="n">
         <v>46071</v>
       </c>
     </row>
@@ -1687,13 +1843,13 @@
         <v>46071</v>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -2211,7 +2367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N256"/>
+  <dimension ref="A1:N259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9825,26 +9981,26 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Innovate Funding Service</t>
+          <t>Innovate UK Business Connect</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Future Leaders Fellowships: Round 10, business and non-academic</t>
+          <t>iX Challenge - Enabling regional carbon dioxide utilisation in Southwest Wales through geospatial intelligence</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2058/overview/0f904547-f415-4fb9-94a7-0701c38a2ba1</t>
+          <t>https://iuk-business-connect.org.uk/opportunities/ix-challenge-enabling-regional-carbon-dioxide-utilisation-southwest-wales/</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>2025-06-14 08:41</t>
+          <t>2026-02-24 10:36</t>
         </is>
       </c>
       <c r="E152" s="1" t="n">
-        <v>45822.36180555556</v>
+        <v>46077.44166666667</v>
       </c>
       <c r="F152" t="b">
         <v>1</v>
@@ -9853,23 +10009,29 @@
       <c r="H152" t="b">
         <v>0</v>
       </c>
-      <c r="I152" t="inlineStr"/>
-      <c r="J152" t="inlineStr"/>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>24/02/2026</t>
+        </is>
+      </c>
+      <c r="J152" s="1" t="n">
+        <v>46077</v>
+      </c>
       <c r="K152" t="inlineStr">
         <is>
-          <t>Wednesday 5 November 2025 11:00am</t>
+          <t>23/04/2026                              23:59</t>
         </is>
       </c>
       <c r="L152" s="1" t="n">
-        <v>45966.45833333334</v>
+        <v>46135.99930555555</v>
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>£3.0 million</t>
+          <t>£25,000</t>
         </is>
       </c>
       <c r="N152" s="1" t="n">
-        <v>45819</v>
+        <v>46071</v>
       </c>
     </row>
     <row r="153">
@@ -9880,12 +10042,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>ADOPT Facilitator Support Grant: Round 2</t>
+          <t>Future Leaders Fellowships: Round 10, business and non-academic</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2223/overview/4e423e05-3228-45e3-9cfe-0b39d1227307</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2058/overview/0f904547-f415-4fb9-94a7-0701c38a2ba1</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -9907,15 +10069,15 @@
       <c r="J153" t="inlineStr"/>
       <c r="K153" t="inlineStr">
         <is>
-          <t>Thursday 24 July 2025 11:00am</t>
+          <t>Wednesday 5 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L153" s="1" t="n">
-        <v>45862.45833333334</v>
+        <v>45966.45833333334</v>
       </c>
       <c r="M153" t="inlineStr">
         <is>
-          <t>£2,500</t>
+          <t>£3.0 million</t>
         </is>
       </c>
       <c r="N153" s="1" t="n">
@@ -9930,12 +10092,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>MSI Improving energy or resource efficiency in manufacturing FS</t>
+          <t>ADOPT Facilitator Support Grant: Round 2</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2225/overview/c43ef163-3872-4178-b80d-88c406691610</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2223/overview/4e423e05-3228-45e3-9cfe-0b39d1227307</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -9957,15 +10119,15 @@
       <c r="J154" t="inlineStr"/>
       <c r="K154" t="inlineStr">
         <is>
-          <t>Wednesday 2 July 2025 11:00am</t>
+          <t>Thursday 24 July 2025 11:00am</t>
         </is>
       </c>
       <c r="L154" s="1" t="n">
-        <v>45840.45833333334</v>
+        <v>45862.45833333334</v>
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£2,500</t>
         </is>
       </c>
       <c r="N154" s="1" t="n">
@@ -9980,12 +10142,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>New Innovators in Marine and Maritime, Great South West</t>
+          <t>MSI Improving energy or resource efficiency in manufacturing FS</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2215/overview/67b86d6c-bab9-4a01-aacc-3da2e57edc99</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2225/overview/c43ef163-3872-4178-b80d-88c406691610</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -10015,7 +10177,7 @@
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>£50,000</t>
+          <t>£100,000</t>
         </is>
       </c>
       <c r="N155" s="1" t="n">
@@ -10030,12 +10192,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Commercialising Knowledge Assets Fund (CKAF) Autumn</t>
+          <t>New Innovators in Marine and Maritime, Great South West</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2217/overview/c555f64e-5485-4e49-89b8-32d61fac4ff0</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2215/overview/67b86d6c-bab9-4a01-aacc-3da2e57edc99</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -10057,15 +10219,15 @@
       <c r="J156" t="inlineStr"/>
       <c r="K156" t="inlineStr">
         <is>
-          <t>Thursday 4 September 2025 11:00am</t>
+          <t>Wednesday 2 July 2025 11:00am</t>
         </is>
       </c>
       <c r="L156" s="1" t="n">
-        <v>45904.45833333334</v>
+        <v>45840.45833333334</v>
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>£250,000</t>
+          <t>£50,000</t>
         </is>
       </c>
       <c r="N156" s="1" t="n">
@@ -10080,12 +10242,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>ATI Programme strategic batch: EoI – June 2025</t>
+          <t>Commercialising Knowledge Assets Fund (CKAF) Autumn</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2218/overview/a45dcc8a-b621-4a79-9e4d-046e19b6b1e9</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2217/overview/c555f64e-5485-4e49-89b8-32d61fac4ff0</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -10107,13 +10269,17 @@
       <c r="J157" t="inlineStr"/>
       <c r="K157" t="inlineStr">
         <is>
-          <t>Wednesday 18 June 2025 11:00am</t>
+          <t>Thursday 4 September 2025 11:00am</t>
         </is>
       </c>
       <c r="L157" s="1" t="n">
-        <v>45826.45833333334</v>
-      </c>
-      <c r="M157" t="inlineStr"/>
+        <v>45904.45833333334</v>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>£250,000</t>
+        </is>
+      </c>
       <c r="N157" s="1" t="n">
         <v>45819</v>
       </c>
@@ -10126,12 +10292,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Defra Farming Innovation Investor Partnership</t>
+          <t>ATI Programme strategic batch: EoI – June 2025</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2207/overview/05e5263b-75a1-49a0-87f0-261541af0840</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2218/overview/a45dcc8a-b621-4a79-9e4d-046e19b6b1e9</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -10153,17 +10319,13 @@
       <c r="J158" t="inlineStr"/>
       <c r="K158" t="inlineStr">
         <is>
-          <t>Wednesday 2 July 2025 11:00am</t>
+          <t>Wednesday 18 June 2025 11:00am</t>
         </is>
       </c>
       <c r="L158" s="1" t="n">
-        <v>45840.45833333334</v>
-      </c>
-      <c r="M158" t="inlineStr">
-        <is>
-          <t>£3.0 million</t>
-        </is>
-      </c>
+        <v>45826.45833333334</v>
+      </c>
+      <c r="M158" t="inlineStr"/>
       <c r="N158" s="1" t="n">
         <v>45819</v>
       </c>
@@ -10176,12 +10338,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Ofgem Strategic Innovation Fund Round 5 Discovery C3</t>
+          <t>Defra Farming Innovation Investor Partnership</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2204/overview/9da241b9-1fd8-49fb-b8d0-4a81a637b3b5</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2207/overview/05e5263b-75a1-49a0-87f0-261541af0840</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -10203,15 +10365,15 @@
       <c r="J159" t="inlineStr"/>
       <c r="K159" t="inlineStr">
         <is>
-          <t>Wednesday 25 June 2025 11:00am</t>
+          <t>Wednesday 2 July 2025 11:00am</t>
         </is>
       </c>
       <c r="L159" s="1" t="n">
-        <v>45833.45833333334</v>
+        <v>45840.45833333334</v>
       </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t>£150,000</t>
+          <t>£3.0 million</t>
         </is>
       </c>
       <c r="N159" s="1" t="n">
@@ -10226,12 +10388,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Ofgem Strategic Innovation Fund Round 4 Discovery C3</t>
+          <t>Ofgem Strategic Innovation Fund Round 5 Discovery C3</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2200/overview/0f0721c8-5a37-4046-8e4f-7649194e8adc</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2204/overview/9da241b9-1fd8-49fb-b8d0-4a81a637b3b5</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -10276,12 +10438,12 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: Scaling community initiatives in diet and exercise</t>
+          <t>Ofgem Strategic Innovation Fund Round 4 Discovery C3</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2191/overview/6a097cf8-8f81-495d-b56f-3f240cfde64c</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2200/overview/0f0721c8-5a37-4046-8e4f-7649194e8adc</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -10303,15 +10465,15 @@
       <c r="J161" t="inlineStr"/>
       <c r="K161" t="inlineStr">
         <is>
-          <t>Wednesday 18 June 2025 11:00am</t>
+          <t>Wednesday 25 June 2025 11:00am</t>
         </is>
       </c>
       <c r="L161" s="1" t="n">
-        <v>45826.45833333334</v>
+        <v>45833.45833333334</v>
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>£250,000</t>
+          <t>£150,000</t>
         </is>
       </c>
       <c r="N161" s="1" t="n">
@@ -10326,12 +10488,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: Quantum Sensors and PNT Missions Primer</t>
+          <t>Contracts for Innovation: Scaling community initiatives in diet and exercise</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2209/overview/28f8801b-a8b3-48c8-8c81-64d75341b81d</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2191/overview/6a097cf8-8f81-495d-b56f-3f240cfde64c</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -10353,15 +10515,15 @@
       <c r="J162" t="inlineStr"/>
       <c r="K162" t="inlineStr">
         <is>
-          <t>Wednesday 2 July 2025 11:00am</t>
+          <t>Wednesday 18 June 2025 11:00am</t>
         </is>
       </c>
       <c r="L162" s="1" t="n">
-        <v>45840.45833333334</v>
+        <v>45826.45833333334</v>
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>£1.5 million</t>
+          <t>£250,000</t>
         </is>
       </c>
       <c r="N162" s="1" t="n">
@@ -10376,12 +10538,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: Net Zero Living Tech Trials, phase 3</t>
+          <t>Contracts for Innovation: Quantum Sensors and PNT Missions Primer</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2189/overview/a59ac38e-662b-49a5-b7f9-a44c2cc38c61</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2209/overview/28f8801b-a8b3-48c8-8c81-64d75341b81d</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -10403,15 +10565,15 @@
       <c r="J163" t="inlineStr"/>
       <c r="K163" t="inlineStr">
         <is>
-          <t>Wednesday 25 June 2025 11:00am</t>
+          <t>Wednesday 2 July 2025 11:00am</t>
         </is>
       </c>
       <c r="L163" s="1" t="n">
-        <v>45833.45833333334</v>
+        <v>45840.45833333334</v>
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£1.5 million</t>
         </is>
       </c>
       <c r="N163" s="1" t="n">
@@ -10426,12 +10588,12 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: Clean Air, Phase 3</t>
+          <t>Contracts for Innovation: Net Zero Living Tech Trials, phase 3</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2181/overview/02aad9d2-c984-4bd5-a3f6-80f25ec62870</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2189/overview/a59ac38e-662b-49a5-b7f9-a44c2cc38c61</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -10476,12 +10638,12 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: DSbD Advancing CHERI Tools and software</t>
+          <t>Contracts for Innovation: Clean Air, Phase 3</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2194/overview/91c68630-20eb-4247-8296-ae1737637756</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2181/overview/02aad9d2-c984-4bd5-a3f6-80f25ec62870</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -10503,15 +10665,15 @@
       <c r="J165" t="inlineStr"/>
       <c r="K165" t="inlineStr">
         <is>
-          <t>Wednesday 18 June 2025 11:00am</t>
+          <t>Wednesday 25 June 2025 11:00am</t>
         </is>
       </c>
       <c r="L165" s="1" t="n">
-        <v>45826.45833333334</v>
+        <v>45833.45833333334</v>
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>£3.0 million</t>
+          <t>£100,000</t>
         </is>
       </c>
       <c r="N165" s="1" t="n">
@@ -10526,12 +10688,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: DSbD Advancing CHERI RISC-V Devices</t>
+          <t>Contracts for Innovation: DSbD Advancing CHERI Tools and software</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2198/overview/b2e2fd41-d372-4e33-a6df-8bfefb8de0f9</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2194/overview/91c68630-20eb-4247-8296-ae1737637756</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -10561,7 +10723,7 @@
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>£5.0 million</t>
+          <t>£3.0 million</t>
         </is>
       </c>
       <c r="N166" s="1" t="n">
@@ -10576,12 +10738,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Canada-UK Semiconductors</t>
+          <t>Contracts for Innovation: DSbD Advancing CHERI RISC-V Devices</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2192/overview/3906cbd5-fec2-4c1f-897d-ccab071708b3</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2198/overview/b2e2fd41-d372-4e33-a6df-8bfefb8de0f9</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -10603,15 +10765,15 @@
       <c r="J167" t="inlineStr"/>
       <c r="K167" t="inlineStr">
         <is>
-          <t>Wednesday 15 October 2025 11:00am</t>
+          <t>Wednesday 18 June 2025 11:00am</t>
         </is>
       </c>
       <c r="L167" s="1" t="n">
-        <v>45945.45833333334</v>
+        <v>45826.45833333334</v>
       </c>
       <c r="M167" t="inlineStr">
         <is>
-          <t>£500,000</t>
+          <t>£5.0 million</t>
         </is>
       </c>
       <c r="N167" s="1" t="n">
@@ -10626,12 +10788,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Accelerated Knowledge Transfer 4 (AKT4) Addiction</t>
+          <t>Canada-UK Semiconductors</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2178/overview/2699060f-dd6f-415b-ae47-bead15aa430e</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2192/overview/3906cbd5-fec2-4c1f-897d-ccab071708b3</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -10653,15 +10815,15 @@
       <c r="J168" t="inlineStr"/>
       <c r="K168" t="inlineStr">
         <is>
-          <t>Wednesday 2 July 2025 11:00am</t>
+          <t>Wednesday 15 October 2025 11:00am</t>
         </is>
       </c>
       <c r="L168" s="1" t="n">
-        <v>45840.45833333334</v>
+        <v>45945.45833333334</v>
       </c>
       <c r="M168" t="inlineStr">
         <is>
-          <t>£35,000</t>
+          <t>£500,000</t>
         </is>
       </c>
       <c r="N168" s="1" t="n">
@@ -10676,12 +10838,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Innovate UK innovation loans future economy: Round 21</t>
+          <t>Accelerated Knowledge Transfer 4 (AKT4) Addiction</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2188/overview/20c89a26-2479-4f80-b35a-b62ed3b9b3ce</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2178/overview/2699060f-dd6f-415b-ae47-bead15aa430e</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -10711,7 +10873,7 @@
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>£2.0 million</t>
+          <t>£35,000</t>
         </is>
       </c>
       <c r="N169" s="1" t="n">
@@ -10726,12 +10888,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Farming Futures R&amp;D Fund: Precision Breeding Competition</t>
+          <t>Innovate UK innovation loans future economy: Round 21</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2168/overview/0fef9171-75b0-4f3e-acef-42920e7e5d5e</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2188/overview/20c89a26-2479-4f80-b35a-b62ed3b9b3ce</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -10753,15 +10915,15 @@
       <c r="J170" t="inlineStr"/>
       <c r="K170" t="inlineStr">
         <is>
-          <t>Wednesday 25 June 2025 11:00am</t>
+          <t>Wednesday 2 July 2025 11:00am</t>
         </is>
       </c>
       <c r="L170" s="1" t="n">
-        <v>45833.45833333334</v>
+        <v>45840.45833333334</v>
       </c>
       <c r="M170" t="inlineStr">
         <is>
-          <t>£2.5 million</t>
+          <t>£2.0 million</t>
         </is>
       </c>
       <c r="N170" s="1" t="n">
@@ -10776,12 +10938,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Farming Futures R&amp;D Fund: low emissions farming</t>
+          <t>Farming Futures R&amp;D Fund: Precision Breeding Competition</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2169/overview/64b0d550-3f46-4ab4-a0cd-5fa7ac488cb6</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2168/overview/0fef9171-75b0-4f3e-acef-42920e7e5d5e</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -10826,12 +10988,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Investor Partnerships: Clean Energy and Climate Technologies</t>
+          <t>Farming Futures R&amp;D Fund: low emissions farming</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2175/overview/7487b4f1-51e6-4f15-a4c8-f103559d14bb</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2169/overview/64b0d550-3f46-4ab4-a0cd-5fa7ac488cb6</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -10853,15 +11015,15 @@
       <c r="J172" t="inlineStr"/>
       <c r="K172" t="inlineStr">
         <is>
-          <t>Wednesday 2 July 2025 11:00am</t>
+          <t>Wednesday 25 June 2025 11:00am</t>
         </is>
       </c>
       <c r="L172" s="1" t="n">
-        <v>45840.45833333334</v>
+        <v>45833.45833333334</v>
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>£2.0 million</t>
+          <t>£2.5 million</t>
         </is>
       </c>
       <c r="N172" s="1" t="n">
@@ -10876,12 +11038,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Full ADOPT Grant: Round 1</t>
+          <t>Investor Partnerships: Clean Energy and Climate Technologies</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2162/overview/c35de0a9-5072-4142-8a52-1cdce8ef3871</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2175/overview/7487b4f1-51e6-4f15-a4c8-f103559d14bb</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -10903,15 +11065,15 @@
       <c r="J173" t="inlineStr"/>
       <c r="K173" t="inlineStr">
         <is>
-          <t>Wednesday 25 June 2025 11:00am</t>
+          <t>Wednesday 2 July 2025 11:00am</t>
         </is>
       </c>
       <c r="L173" s="1" t="n">
-        <v>45833.45833333334</v>
+        <v>45840.45833333334</v>
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£2.0 million</t>
         </is>
       </c>
       <c r="N173" s="1" t="n">
@@ -10926,12 +11088,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Horizon Europe Guarantee - EIT KICs 2023</t>
+          <t>Full ADOPT Grant: Round 1</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/1585/overview/32135a71-171a-46bf-ad56-e2e65a1a3574</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2162/overview/c35de0a9-5072-4142-8a52-1cdce8ef3871</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -10953,11 +11115,17 @@
       <c r="J174" t="inlineStr"/>
       <c r="K174" t="inlineStr">
         <is>
-          <t>Thursday 27 November 2025 4:00pm</t>
-        </is>
-      </c>
-      <c r="L174" t="inlineStr"/>
-      <c r="M174" t="inlineStr"/>
+          <t>Wednesday 25 June 2025 11:00am</t>
+        </is>
+      </c>
+      <c r="L174" s="1" t="n">
+        <v>45833.45833333334</v>
+      </c>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>£100,000</t>
+        </is>
+      </c>
       <c r="N174" s="1" t="n">
         <v>45819</v>
       </c>
@@ -10970,12 +11138,12 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Horizon Europe Guarantee Extension</t>
+          <t>Horizon Europe Guarantee - EIT KICs 2023</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/1389/overview/b900fdc4-c48d-4d8a-8733-ce4ca210ae9a</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/1585/overview/32135a71-171a-46bf-ad56-e2e65a1a3574</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -11014,21 +11182,21 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Knowledge Transfer Partnership (KTP): 2025 – 2026 Round 3</t>
+          <t>Horizon Europe Guarantee Extension</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2184/overview/c599b17c-e13a-4e13-995e-53cc4d4508a1</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/1389/overview/b900fdc4-c48d-4d8a-8733-ce4ca210ae9a</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>2025-06-16 22:04</t>
+          <t>2025-06-14 08:41</t>
         </is>
       </c>
       <c r="E176" s="1" t="n">
-        <v>45824.91944444444</v>
+        <v>45822.36180555556</v>
       </c>
       <c r="F176" t="b">
         <v>1</v>
@@ -11041,17 +11209,11 @@
       <c r="J176" t="inlineStr"/>
       <c r="K176" t="inlineStr">
         <is>
-          <t>Wednesday 17 September 2025 11:00am</t>
-        </is>
-      </c>
-      <c r="L176" s="1" t="n">
-        <v>45917.45833333334</v>
-      </c>
-      <c r="M176" t="inlineStr">
-        <is>
-          <t>£8,500</t>
-        </is>
-      </c>
+          <t>Thursday 27 November 2025 4:00pm</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr"/>
+      <c r="M176" t="inlineStr"/>
       <c r="N176" s="1" t="n">
         <v>45819</v>
       </c>
@@ -11064,21 +11226,21 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Agri-tech and food technology, Mid and North Wales - CRD</t>
+          <t>Knowledge Transfer Partnership (KTP): 2025 – 2026 Round 3</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2212/overview/4411087f-2a92-4aed-b735-d1a813376bec</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2184/overview/c599b17c-e13a-4e13-995e-53cc4d4508a1</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>2025-06-26 08:52</t>
+          <t>2025-06-16 22:04</t>
         </is>
       </c>
       <c r="E177" s="1" t="n">
-        <v>45834.36944444444</v>
+        <v>45824.91944444444</v>
       </c>
       <c r="F177" t="b">
         <v>1</v>
@@ -11091,19 +11253,19 @@
       <c r="J177" t="inlineStr"/>
       <c r="K177" t="inlineStr">
         <is>
-          <t>Wednesday 20 August 2025 11:00am</t>
+          <t>Wednesday 17 September 2025 11:00am</t>
         </is>
       </c>
       <c r="L177" s="1" t="n">
-        <v>45889.45833333334</v>
+        <v>45917.45833333334</v>
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>£500,000</t>
+          <t>£8,500</t>
         </is>
       </c>
       <c r="N177" s="1" t="n">
-        <v>45833</v>
+        <v>45819</v>
       </c>
     </row>
     <row r="178">
@@ -11114,12 +11276,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Full ADOPT Grant Round 2</t>
+          <t>Agri-tech and food technology, Mid and North Wales - CRD</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2222/overview/c3d5b2f9-e4d4-4ddc-99a2-589904ac3d42</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2212/overview/4411087f-2a92-4aed-b735-d1a813376bec</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -11149,7 +11311,7 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£500,000</t>
         </is>
       </c>
       <c r="N178" s="1" t="n">
@@ -11164,21 +11326,21 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Innovate UK Innovation Loans Round 22</t>
+          <t>Full ADOPT Grant Round 2</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2236/overview/70cbae59-4e67-4626-8cb0-6bbbfc0cf6b7</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2222/overview/c3d5b2f9-e4d4-4ddc-99a2-589904ac3d42</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>2025-07-03 08:52</t>
+          <t>2025-06-26 08:52</t>
         </is>
       </c>
       <c r="E179" s="1" t="n">
-        <v>45841.36944444444</v>
+        <v>45834.36944444444</v>
       </c>
       <c r="F179" t="b">
         <v>1</v>
@@ -11191,19 +11353,19 @@
       <c r="J179" t="inlineStr"/>
       <c r="K179" t="inlineStr">
         <is>
-          <t>Wednesday 27 August 2025 11:00am</t>
+          <t>Wednesday 20 August 2025 11:00am</t>
         </is>
       </c>
       <c r="L179" s="1" t="n">
-        <v>45896.45833333334</v>
+        <v>45889.45833333334</v>
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>£5.0 million</t>
+          <t>£100,000</t>
         </is>
       </c>
       <c r="N179" s="1" t="n">
-        <v>45840</v>
+        <v>45833</v>
       </c>
     </row>
     <row r="180">
@@ -11214,21 +11376,21 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Growth Catalyst Early Stage: New Innovators</t>
+          <t>Innovate UK Innovation Loans Round 22</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2220/overview/bcfd2780-f307-4434-be32-46889a239024</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2236/overview/70cbae59-4e67-4626-8cb0-6bbbfc0cf6b7</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>2025-07-07 08:54</t>
+          <t>2025-07-03 08:52</t>
         </is>
       </c>
       <c r="E180" s="1" t="n">
-        <v>45845.37083333333</v>
+        <v>45841.36944444444</v>
       </c>
       <c r="F180" t="b">
         <v>1</v>
@@ -11241,15 +11403,15 @@
       <c r="J180" t="inlineStr"/>
       <c r="K180" t="inlineStr">
         <is>
-          <t>Wednesday 6 August 2025 11:00am</t>
+          <t>Wednesday 27 August 2025 11:00am</t>
         </is>
       </c>
       <c r="L180" s="1" t="n">
-        <v>45875.45833333334</v>
+        <v>45896.45833333334</v>
       </c>
       <c r="M180" t="inlineStr">
         <is>
-          <t>£50,000</t>
+          <t>£5.0 million</t>
         </is>
       </c>
       <c r="N180" s="1" t="n">
@@ -11264,12 +11426,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>ATI Programme strategic batch: EoI – July 2025</t>
+          <t>Growth Catalyst Early Stage: New Innovators</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2228/overview/5ccf059d-ae66-4f72-a319-4b12cbd46d1c</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2220/overview/bcfd2780-f307-4434-be32-46889a239024</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -11291,13 +11453,17 @@
       <c r="J181" t="inlineStr"/>
       <c r="K181" t="inlineStr">
         <is>
-          <t>Wednesday 23 July 2025 11:00am</t>
+          <t>Wednesday 6 August 2025 11:00am</t>
         </is>
       </c>
       <c r="L181" s="1" t="n">
-        <v>45861.45833333334</v>
-      </c>
-      <c r="M181" t="inlineStr"/>
+        <v>45875.45833333334</v>
+      </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>£50,000</t>
+        </is>
+      </c>
       <c r="N181" s="1" t="n">
         <v>45840</v>
       </c>
@@ -11310,21 +11476,21 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: Resource Efficient Construction Impacts</t>
+          <t>ATI Programme strategic batch: EoI – July 2025</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2242/overview/51b1338a-0d60-43de-b062-fe7a48a7d42f</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2228/overview/5ccf059d-ae66-4f72-a319-4b12cbd46d1c</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>2025-07-09 08:54</t>
+          <t>2025-07-07 08:54</t>
         </is>
       </c>
       <c r="E182" s="1" t="n">
-        <v>45847.37083333333</v>
+        <v>45845.37083333333</v>
       </c>
       <c r="F182" t="b">
         <v>1</v>
@@ -11337,19 +11503,15 @@
       <c r="J182" t="inlineStr"/>
       <c r="K182" t="inlineStr">
         <is>
-          <t>Wednesday 27 August 2025 11:00am</t>
+          <t>Wednesday 23 July 2025 11:00am</t>
         </is>
       </c>
       <c r="L182" s="1" t="n">
-        <v>45896.45833333334</v>
-      </c>
-      <c r="M182" t="inlineStr">
-        <is>
-          <t>£300,000</t>
-        </is>
-      </c>
+        <v>45861.45833333334</v>
+      </c>
+      <c r="M182" t="inlineStr"/>
       <c r="N182" s="1" t="n">
-        <v>45847</v>
+        <v>45840</v>
       </c>
     </row>
     <row r="183">
@@ -11360,12 +11522,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: Resource Efficient Chemicals Impacts</t>
+          <t>Contracts for Innovation: Resource Efficient Construction Impacts</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2240/overview/10f28eca-01f0-4abf-8e0c-998151fe747b</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2242/overview/51b1338a-0d60-43de-b062-fe7a48a7d42f</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -11410,12 +11572,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: Resource Efficient Automotive Impacts</t>
+          <t>Contracts for Innovation: Resource Efficient Chemicals Impacts</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2241/overview/baec7aff-ca8b-456c-9e4d-d6eb9621a988</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2240/overview/10f28eca-01f0-4abf-8e0c-998151fe747b</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -11460,12 +11622,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Future Flight: Regional Demonstrator 2</t>
+          <t>Contracts for Innovation: Resource Efficient Automotive Impacts</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2239/overview/7c5a9acd-4b31-414a-8e35-20dd1df3a2a1</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2241/overview/baec7aff-ca8b-456c-9e4d-d6eb9621a988</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -11487,15 +11649,15 @@
       <c r="J185" t="inlineStr"/>
       <c r="K185" t="inlineStr">
         <is>
-          <t>Thursday 17 July 2025 11:00am</t>
+          <t>Wednesday 27 August 2025 11:00am</t>
         </is>
       </c>
       <c r="L185" s="1" t="n">
-        <v>45855.45833333334</v>
+        <v>45896.45833333334</v>
       </c>
       <c r="M185" t="inlineStr">
         <is>
-          <t>£200,000</t>
+          <t>£300,000</t>
         </is>
       </c>
       <c r="N185" s="1" t="n">
@@ -11510,21 +11672,21 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>DRIVE35 Scale-up: Feasibility Studies</t>
+          <t>Future Flight: Regional Demonstrator 2</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2247/overview/53da287a-c141-48d2-a3eb-f854e14c6578</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2239/overview/7c5a9acd-4b31-414a-8e35-20dd1df3a2a1</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>2025-07-15 08:20</t>
+          <t>2025-07-09 08:54</t>
         </is>
       </c>
       <c r="E186" s="1" t="n">
-        <v>45853.34722222222</v>
+        <v>45847.37083333333</v>
       </c>
       <c r="F186" t="b">
         <v>1</v>
@@ -11537,15 +11699,15 @@
       <c r="J186" t="inlineStr"/>
       <c r="K186" t="inlineStr">
         <is>
-          <t>Wednesday 3 September 2025 11:00am</t>
+          <t>Thursday 17 July 2025 11:00am</t>
         </is>
       </c>
       <c r="L186" s="1" t="n">
-        <v>45903.45833333334</v>
+        <v>45855.45833333334</v>
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>£750,000</t>
+          <t>£200,000</t>
         </is>
       </c>
       <c r="N186" s="1" t="n">
@@ -11560,12 +11722,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>DRIVE35 Innovation Fund: Demonstrate</t>
+          <t>DRIVE35 Scale-up: Feasibility Studies</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2245/overview/777781a3-f181-42b3-a05e-86b96754f28d</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2247/overview/53da287a-c141-48d2-a3eb-f854e14c6578</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -11587,15 +11749,15 @@
       <c r="J187" t="inlineStr"/>
       <c r="K187" t="inlineStr">
         <is>
-          <t>Wednesday 1 October 2025 11:00am</t>
+          <t>Wednesday 3 September 2025 11:00am</t>
         </is>
       </c>
       <c r="L187" s="1" t="n">
-        <v>45931.45833333334</v>
+        <v>45903.45833333334</v>
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>£1.5 million</t>
+          <t>£750,000</t>
         </is>
       </c>
       <c r="N187" s="1" t="n">
@@ -11610,12 +11772,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>DRIVE35 Innovation Fund: Collaborate</t>
+          <t>DRIVE35 Innovation Fund: Demonstrate</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2244/overview/84f81488-4936-4551-a315-7ec40cf1065d</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2245/overview/777781a3-f181-42b3-a05e-86b96754f28d</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -11645,7 +11807,7 @@
       </c>
       <c r="M188" t="inlineStr">
         <is>
-          <t>£25.0 million</t>
+          <t>£1.5 million</t>
         </is>
       </c>
       <c r="N188" s="1" t="n">
@@ -11660,21 +11822,21 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>ADOPT Facilitator Support Grant: Round 3</t>
+          <t>DRIVE35 Innovation Fund: Collaborate</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2251/overview/f40e861a-c7f6-4597-ac5d-2e8d1b4f59f8</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2244/overview/84f81488-4936-4551-a315-7ec40cf1065d</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>2025-07-25 08:20</t>
+          <t>2025-07-15 08:20</t>
         </is>
       </c>
       <c r="E189" s="1" t="n">
-        <v>45863.34722222222</v>
+        <v>45853.34722222222</v>
       </c>
       <c r="F189" t="b">
         <v>1</v>
@@ -11687,19 +11849,19 @@
       <c r="J189" t="inlineStr"/>
       <c r="K189" t="inlineStr">
         <is>
-          <t>Wednesday 3 September 2025 11:00am</t>
+          <t>Wednesday 1 October 2025 11:00am</t>
         </is>
       </c>
       <c r="L189" s="1" t="n">
-        <v>45903.45833333334</v>
+        <v>45931.45833333334</v>
       </c>
       <c r="M189" t="inlineStr">
         <is>
-          <t>£2,500</t>
+          <t>£25.0 million</t>
         </is>
       </c>
       <c r="N189" s="1" t="n">
-        <v>45861</v>
+        <v>45847</v>
       </c>
     </row>
     <row r="190">
@@ -11710,21 +11872,21 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Sovereign AI - Proof of concept</t>
+          <t>ADOPT Facilitator Support Grant: Round 3</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2259/overview/9061ddb2-fa12-45c9-8691-d36649c96e9c</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2251/overview/f40e861a-c7f6-4597-ac5d-2e8d1b4f59f8</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>2025-08-07 08:21</t>
+          <t>2025-07-25 08:20</t>
         </is>
       </c>
       <c r="E190" s="1" t="n">
-        <v>45876.34791666667</v>
+        <v>45863.34722222222</v>
       </c>
       <c r="F190" t="b">
         <v>1</v>
@@ -11737,19 +11899,19 @@
       <c r="J190" t="inlineStr"/>
       <c r="K190" t="inlineStr">
         <is>
-          <t>Wednesday 10 September 2025 11:00am</t>
+          <t>Wednesday 3 September 2025 11:00am</t>
         </is>
       </c>
       <c r="L190" s="1" t="n">
-        <v>45910.45833333334</v>
+        <v>45903.45833333334</v>
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>£120,000</t>
+          <t>£2,500</t>
         </is>
       </c>
       <c r="N190" s="1" t="n">
-        <v>45875</v>
+        <v>45861</v>
       </c>
     </row>
     <row r="191">
@@ -11760,21 +11922,21 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Obesity Pathway Innovation Programme (OPIP): Strand 3</t>
+          <t>Sovereign AI - Proof of concept</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2186/overview/e51c18bc-21b3-450d-bdbc-2f43dad3b268</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2259/overview/9061ddb2-fa12-45c9-8691-d36649c96e9c</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>2025-08-14 08:20</t>
+          <t>2025-08-07 08:21</t>
         </is>
       </c>
       <c r="E191" s="1" t="n">
-        <v>45883.34722222222</v>
+        <v>45876.34791666667</v>
       </c>
       <c r="F191" t="b">
         <v>1</v>
@@ -11787,19 +11949,19 @@
       <c r="J191" t="inlineStr"/>
       <c r="K191" t="inlineStr">
         <is>
-          <t>Wednesday 19 November 2025 11:00am</t>
+          <t>Wednesday 10 September 2025 11:00am</t>
         </is>
       </c>
       <c r="L191" s="1" t="n">
-        <v>45980.45833333334</v>
+        <v>45910.45833333334</v>
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>£8.0 million</t>
+          <t>£120,000</t>
         </is>
       </c>
       <c r="N191" s="1" t="n">
-        <v>45882</v>
+        <v>45875</v>
       </c>
     </row>
     <row r="192">
@@ -11810,12 +11972,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Obesity Pathway Innovation Programme (OPIP): Strand 2</t>
+          <t>Obesity Pathway Innovation Programme (OPIP): Strand 3</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2185/overview/d5b2aeb3-c2e4-4d78-9be3-f1d9919b0956</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2186/overview/e51c18bc-21b3-450d-bdbc-2f43dad3b268</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -11845,7 +12007,7 @@
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t>£4.5 million</t>
+          <t>£8.0 million</t>
         </is>
       </c>
       <c r="N192" s="1" t="n">
@@ -11860,12 +12022,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Obesity Pathway Innovation Programme (OPIP): Strand 1</t>
+          <t>Obesity Pathway Innovation Programme (OPIP): Strand 2</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2177/overview/696c1e3c-589d-4c37-8958-6255d1dc125a</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2185/overview/d5b2aeb3-c2e4-4d78-9be3-f1d9919b0956</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -11895,7 +12057,7 @@
       </c>
       <c r="M193" t="inlineStr">
         <is>
-          <t>£3.5 million</t>
+          <t>£4.5 million</t>
         </is>
       </c>
       <c r="N193" s="1" t="n">
@@ -11910,21 +12072,21 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Analysis for Innovators: National Physical Laboratory Stage 1</t>
+          <t>Obesity Pathway Innovation Programme (OPIP): Strand 1</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2266/overview/2fcad3ee-b5d6-4f01-8b1a-0e1af3c93023</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2177/overview/696c1e3c-589d-4c37-8958-6255d1dc125a</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>2025-08-26 08:20</t>
+          <t>2025-08-14 08:20</t>
         </is>
       </c>
       <c r="E194" s="1" t="n">
-        <v>45895.34722222222</v>
+        <v>45883.34722222222</v>
       </c>
       <c r="F194" t="b">
         <v>1</v>
@@ -11937,19 +12099,19 @@
       <c r="J194" t="inlineStr"/>
       <c r="K194" t="inlineStr">
         <is>
-          <t>Wednesday 10 September 2025 11:00am</t>
+          <t>Wednesday 19 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L194" s="1" t="n">
-        <v>45910.45833333334</v>
+        <v>45980.45833333334</v>
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£3.5 million</t>
         </is>
       </c>
       <c r="N194" s="1" t="n">
-        <v>45889</v>
+        <v>45882</v>
       </c>
     </row>
     <row r="195">
@@ -11960,21 +12122,21 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Full ADOPT Grant Round 3</t>
+          <t>Analysis for Innovators: National Physical Laboratory Stage 1</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2265/overview/fae182db-d9e5-4173-bb59-8fde361ccad4</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2266/overview/2fcad3ee-b5d6-4f01-8b1a-0e1af3c93023</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>2025-08-27 08:18</t>
+          <t>2025-08-26 08:20</t>
         </is>
       </c>
       <c r="E195" s="1" t="n">
-        <v>45896.34583333333</v>
+        <v>45895.34722222222</v>
       </c>
       <c r="F195" t="b">
         <v>1</v>
@@ -11987,11 +12149,11 @@
       <c r="J195" t="inlineStr"/>
       <c r="K195" t="inlineStr">
         <is>
-          <t>Wednesday 15 October 2025 11:00am</t>
+          <t>Wednesday 10 September 2025 11:00am</t>
         </is>
       </c>
       <c r="L195" s="1" t="n">
-        <v>45945.45833333334</v>
+        <v>45910.45833333334</v>
       </c>
       <c r="M195" t="inlineStr">
         <is>
@@ -11999,7 +12161,7 @@
         </is>
       </c>
       <c r="N195" s="1" t="n">
-        <v>45896</v>
+        <v>45889</v>
       </c>
     </row>
     <row r="196">
@@ -12010,21 +12172,21 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>ATI Programme strategic batch: EoI – September 2025</t>
+          <t>Full ADOPT Grant Round 3</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2273/overview/b30df196-a9a2-4e53-85e1-e3e6aaa5c5b7</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2265/overview/fae182db-d9e5-4173-bb59-8fde361ccad4</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>2025-09-01 08:20</t>
+          <t>2025-08-27 08:18</t>
         </is>
       </c>
       <c r="E196" s="1" t="n">
-        <v>45901.34722222222</v>
+        <v>45896.34583333333</v>
       </c>
       <c r="F196" t="b">
         <v>1</v>
@@ -12037,13 +12199,17 @@
       <c r="J196" t="inlineStr"/>
       <c r="K196" t="inlineStr">
         <is>
-          <t>Wednesday 17 September 2025 11:00am</t>
+          <t>Wednesday 15 October 2025 11:00am</t>
         </is>
       </c>
       <c r="L196" s="1" t="n">
-        <v>45917.45833333334</v>
-      </c>
-      <c r="M196" t="inlineStr"/>
+        <v>45945.45833333334</v>
+      </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>£100,000</t>
+        </is>
+      </c>
       <c r="N196" s="1" t="n">
         <v>45896</v>
       </c>
@@ -12056,21 +12222,21 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Farming Innovation Programme: Small R&amp;D Partnership Projects Rd 4</t>
+          <t>ATI Programme strategic batch: EoI – September 2025</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2010/overview/bcd5cf06-313c-4197-ae47-0035f674717f</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2273/overview/b30df196-a9a2-4e53-85e1-e3e6aaa5c5b7</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>2025-09-02 08:19</t>
+          <t>2025-09-01 08:20</t>
         </is>
       </c>
       <c r="E197" s="1" t="n">
-        <v>45902.34652777778</v>
+        <v>45901.34722222222</v>
       </c>
       <c r="F197" t="b">
         <v>1</v>
@@ -12083,17 +12249,13 @@
       <c r="J197" t="inlineStr"/>
       <c r="K197" t="inlineStr">
         <is>
-          <t>Wednesday 5 November 2025 11:00am</t>
+          <t>Wednesday 17 September 2025 11:00am</t>
         </is>
       </c>
       <c r="L197" s="1" t="n">
-        <v>45966.45833333334</v>
-      </c>
-      <c r="M197" t="inlineStr">
-        <is>
-          <t>£3.0 million</t>
-        </is>
-      </c>
+        <v>45917.45833333334</v>
+      </c>
+      <c r="M197" t="inlineStr"/>
       <c r="N197" s="1" t="n">
         <v>45896</v>
       </c>
@@ -12106,21 +12268,21 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>ADOPT Facilitator Support Grant: Round 4</t>
+          <t>Farming Innovation Programme: Small R&amp;D Partnership Projects Rd 4</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2277/overview/7386173a-c074-4617-b7d0-f54f3a458247</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2010/overview/bcd5cf06-313c-4197-ae47-0035f674717f</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>2025-09-04 08:18</t>
+          <t>2025-09-02 08:19</t>
         </is>
       </c>
       <c r="E198" s="1" t="n">
-        <v>45904.34583333333</v>
+        <v>45902.34652777778</v>
       </c>
       <c r="F198" t="b">
         <v>1</v>
@@ -12133,19 +12295,19 @@
       <c r="J198" t="inlineStr"/>
       <c r="K198" t="inlineStr">
         <is>
-          <t>Wednesday 15 October 2025 11:00am</t>
+          <t>Wednesday 5 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L198" s="1" t="n">
-        <v>45945.45833333334</v>
+        <v>45966.45833333334</v>
       </c>
       <c r="M198" t="inlineStr">
         <is>
-          <t>£2,500</t>
+          <t>£3.0 million</t>
         </is>
       </c>
       <c r="N198" s="1" t="n">
-        <v>45903</v>
+        <v>45896</v>
       </c>
     </row>
     <row r="199">
@@ -12156,21 +12318,21 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Innovate UK Innovation Loans Round 23</t>
+          <t>ADOPT Facilitator Support Grant: Round 4</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2275/overview/dec9b656-5f30-414e-a169-e11e17d04896</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2277/overview/7386173a-c074-4617-b7d0-f54f3a458247</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>2025-09-05 08:18</t>
+          <t>2025-09-04 08:18</t>
         </is>
       </c>
       <c r="E199" s="1" t="n">
-        <v>45905.34583333333</v>
+        <v>45904.34583333333</v>
       </c>
       <c r="F199" t="b">
         <v>1</v>
@@ -12183,15 +12345,15 @@
       <c r="J199" t="inlineStr"/>
       <c r="K199" t="inlineStr">
         <is>
-          <t>Wednesday 22 October 2025 11:00am</t>
+          <t>Wednesday 15 October 2025 11:00am</t>
         </is>
       </c>
       <c r="L199" s="1" t="n">
-        <v>45952.45833333334</v>
+        <v>45945.45833333334</v>
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>£5.0 million</t>
+          <t>£2,500</t>
         </is>
       </c>
       <c r="N199" s="1" t="n">
@@ -12206,21 +12368,21 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>UK-Netherlands Co-Innovation and Testbeds Pilot for Quantum Tech</t>
+          <t>Innovate UK Innovation Loans Round 23</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2288/overview/d547d84e-d652-4ed6-9c85-b12ab8d785d2</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2275/overview/dec9b656-5f30-414e-a169-e11e17d04896</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>2025-09-12 08:17</t>
+          <t>2025-09-05 08:18</t>
         </is>
       </c>
       <c r="E200" s="1" t="n">
-        <v>45912.34513888889</v>
+        <v>45905.34583333333</v>
       </c>
       <c r="F200" t="b">
         <v>1</v>
@@ -12233,19 +12395,19 @@
       <c r="J200" t="inlineStr"/>
       <c r="K200" t="inlineStr">
         <is>
-          <t>Tuesday 28 October 2025 11:00am</t>
+          <t>Wednesday 22 October 2025 11:00am</t>
         </is>
       </c>
       <c r="L200" s="1" t="n">
-        <v>45958.45833333334</v>
+        <v>45952.45833333334</v>
       </c>
       <c r="M200" t="inlineStr">
         <is>
-          <t>£300,000</t>
+          <t>£5.0 million</t>
         </is>
       </c>
       <c r="N200" s="1" t="n">
-        <v>45910</v>
+        <v>45903</v>
       </c>
     </row>
     <row r="201">
@@ -12256,21 +12418,21 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: Quantum Technologies for Transport - Phase 1</t>
+          <t>UK-Netherlands Co-Innovation and Testbeds Pilot for Quantum Tech</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2292/overview/cdea3182-7495-4cad-8435-f49882f08ec7</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2288/overview/d547d84e-d652-4ed6-9c85-b12ab8d785d2</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>2025-09-16 08:19</t>
+          <t>2025-09-12 08:17</t>
         </is>
       </c>
       <c r="E201" s="1" t="n">
-        <v>45916.34652777778</v>
+        <v>45912.34513888889</v>
       </c>
       <c r="F201" t="b">
         <v>1</v>
@@ -12283,15 +12445,15 @@
       <c r="J201" t="inlineStr"/>
       <c r="K201" t="inlineStr">
         <is>
-          <t>Wednesday 15 October 2025 11:00am</t>
+          <t>Tuesday 28 October 2025 11:00am</t>
         </is>
       </c>
       <c r="L201" s="1" t="n">
-        <v>45945.45833333334</v>
+        <v>45958.45833333334</v>
       </c>
       <c r="M201" t="inlineStr">
         <is>
-          <t>£40,000</t>
+          <t>£300,000</t>
         </is>
       </c>
       <c r="N201" s="1" t="n">
@@ -12306,21 +12468,21 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>DRIVE35 Scale-up Fund</t>
+          <t>Contracts for Innovation: Quantum Technologies for Transport - Phase 1</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2279/overview/029bd996-9abd-42d9-8134-e2d34e3cfff5</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2292/overview/cdea3182-7495-4cad-8435-f49882f08ec7</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>2025-09-17 08:18</t>
+          <t>2025-09-16 08:19</t>
         </is>
       </c>
       <c r="E202" s="1" t="n">
-        <v>45917.34583333333</v>
+        <v>45916.34652777778</v>
       </c>
       <c r="F202" t="b">
         <v>1</v>
@@ -12333,17 +12495,19 @@
       <c r="J202" t="inlineStr"/>
       <c r="K202" t="inlineStr">
         <is>
-          <t>There is no submission deadline</t>
-        </is>
-      </c>
-      <c r="L202" t="inlineStr"/>
+          <t>Wednesday 15 October 2025 11:00am</t>
+        </is>
+      </c>
+      <c r="L202" s="1" t="n">
+        <v>45945.45833333334</v>
+      </c>
       <c r="M202" t="inlineStr">
         <is>
-          <t>£20.0 million</t>
+          <t>£40,000</t>
         </is>
       </c>
       <c r="N202" s="1" t="n">
-        <v>45917</v>
+        <v>45910</v>
       </c>
     </row>
     <row r="203">
@@ -12354,21 +12518,21 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Commercialising Knowledge Assets Fund (CKAF) Winter</t>
+          <t>DRIVE35 Scale-up Fund</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2295/overview/cdce9dab-263c-444b-9e91-61f13046bd62</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2279/overview/029bd996-9abd-42d9-8134-e2d34e3cfff5</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>2025-09-18 08:17</t>
+          <t>2025-09-17 08:18</t>
         </is>
       </c>
       <c r="E203" s="1" t="n">
-        <v>45918.34513888889</v>
+        <v>45917.34583333333</v>
       </c>
       <c r="F203" t="b">
         <v>1</v>
@@ -12381,15 +12545,13 @@
       <c r="J203" t="inlineStr"/>
       <c r="K203" t="inlineStr">
         <is>
-          <t>Thursday 4 December 2025 11:00am</t>
-        </is>
-      </c>
-      <c r="L203" s="1" t="n">
-        <v>45995.45833333334</v>
-      </c>
+          <t>There is no submission deadline</t>
+        </is>
+      </c>
+      <c r="L203" t="inlineStr"/>
       <c r="M203" t="inlineStr">
         <is>
-          <t>£250,000</t>
+          <t>£20.0 million</t>
         </is>
       </c>
       <c r="N203" s="1" t="n">
@@ -12404,21 +12566,21 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Resource efficiency for resilience and sustainability FS</t>
+          <t>Commercialising Knowledge Assets Fund (CKAF) Winter</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2293/overview/2efee934-8622-4686-bc02-a6ac7fc9e5a6</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2295/overview/cdce9dab-263c-444b-9e91-61f13046bd62</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>2025-09-20 08:16</t>
+          <t>2025-09-18 08:17</t>
         </is>
       </c>
       <c r="E204" s="1" t="n">
-        <v>45920.34444444445</v>
+        <v>45918.34513888889</v>
       </c>
       <c r="F204" t="b">
         <v>1</v>
@@ -12431,15 +12593,15 @@
       <c r="J204" t="inlineStr"/>
       <c r="K204" t="inlineStr">
         <is>
-          <t>Monday 3 November 2025 11:00am</t>
+          <t>Thursday 4 December 2025 11:00am</t>
         </is>
       </c>
       <c r="L204" s="1" t="n">
-        <v>45964.45833333334</v>
+        <v>45995.45833333334</v>
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>£25,000</t>
+          <t>£250,000</t>
         </is>
       </c>
       <c r="N204" s="1" t="n">
@@ -12454,21 +12616,21 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Ofgem Strategic Innovation Fund Round 5 Discovery C4</t>
+          <t>Resource efficiency for resilience and sustainability FS</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2284/overview/aa6bd2b1-f6e1-4e96-bd4c-0557c10779c8</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2293/overview/2efee934-8622-4686-bc02-a6ac7fc9e5a6</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>2025-09-23 08:18</t>
+          <t>2025-09-20 08:16</t>
         </is>
       </c>
       <c r="E205" s="1" t="n">
-        <v>45923.34583333333</v>
+        <v>45920.34444444445</v>
       </c>
       <c r="F205" t="b">
         <v>1</v>
@@ -12481,15 +12643,15 @@
       <c r="J205" t="inlineStr"/>
       <c r="K205" t="inlineStr">
         <is>
-          <t>Wednesday 22 October 2025 11:00am</t>
+          <t>Monday 3 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L205" s="1" t="n">
-        <v>45952.45833333334</v>
+        <v>45964.45833333334</v>
       </c>
       <c r="M205" t="inlineStr">
         <is>
-          <t>£150,000</t>
+          <t>£25,000</t>
         </is>
       </c>
       <c r="N205" s="1" t="n">
@@ -12504,21 +12666,21 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Farming Innovation Programme: Feasibility Round 4</t>
+          <t>Ofgem Strategic Innovation Fund Round 5 Discovery C4</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2006/overview/b67973b5-6d46-4a34-a864-bec1212e3fe0</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2284/overview/aa6bd2b1-f6e1-4e96-bd4c-0557c10779c8</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>2025-09-29 08:20</t>
+          <t>2025-09-23 08:18</t>
         </is>
       </c>
       <c r="E206" s="1" t="n">
-        <v>45929.34722222222</v>
+        <v>45923.34583333333</v>
       </c>
       <c r="F206" t="b">
         <v>1</v>
@@ -12531,19 +12693,19 @@
       <c r="J206" t="inlineStr"/>
       <c r="K206" t="inlineStr">
         <is>
-          <t>Wednesday 3 December 2025 11:00am</t>
+          <t>Wednesday 22 October 2025 11:00am</t>
         </is>
       </c>
       <c r="L206" s="1" t="n">
-        <v>45994.45833333334</v>
+        <v>45952.45833333334</v>
       </c>
       <c r="M206" t="inlineStr">
         <is>
-          <t>£500,000</t>
+          <t>£150,000</t>
         </is>
       </c>
       <c r="N206" s="1" t="n">
-        <v>45924</v>
+        <v>45917</v>
       </c>
     </row>
     <row r="207">
@@ -12554,21 +12716,21 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Eureka GlobalStars Japan 2026</t>
+          <t>Farming Innovation Programme: Feasibility Round 4</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2276/overview/19635c62-dd91-41d8-a90e-547cdb5acbfa</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2006/overview/b67973b5-6d46-4a34-a864-bec1212e3fe0</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>2025-10-03 08:17</t>
+          <t>2025-09-29 08:20</t>
         </is>
       </c>
       <c r="E207" s="1" t="n">
-        <v>45933.34513888889</v>
+        <v>45929.34722222222</v>
       </c>
       <c r="F207" t="b">
         <v>1</v>
@@ -12581,19 +12743,19 @@
       <c r="J207" t="inlineStr"/>
       <c r="K207" t="inlineStr">
         <is>
-          <t>Wednesday 21 January 2026 11:00am</t>
+          <t>Wednesday 3 December 2025 11:00am</t>
         </is>
       </c>
       <c r="L207" s="1" t="n">
-        <v>46043.45833333334</v>
+        <v>45994.45833333334</v>
       </c>
       <c r="M207" t="inlineStr">
         <is>
-          <t>£600,000</t>
+          <t>£500,000</t>
         </is>
       </c>
       <c r="N207" s="1" t="n">
-        <v>45931</v>
+        <v>45924</v>
       </c>
     </row>
     <row r="208">
@@ -12604,21 +12766,21 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>CAM Pathfinder: Feasibility studies 2</t>
+          <t>Eureka GlobalStars Japan 2026</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2307/overview/8eec43e7-96a5-49d1-97e1-3400321160f9</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2276/overview/19635c62-dd91-41d8-a90e-547cdb5acbfa</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>2025-10-10 08:18</t>
+          <t>2025-10-03 08:17</t>
         </is>
       </c>
       <c r="E208" s="1" t="n">
-        <v>45940.34583333333</v>
+        <v>45933.34513888889</v>
       </c>
       <c r="F208" t="b">
         <v>1</v>
@@ -12631,19 +12793,19 @@
       <c r="J208" t="inlineStr"/>
       <c r="K208" t="inlineStr">
         <is>
-          <t>Wednesday 26 November 2025 11:00am</t>
+          <t>Wednesday 21 January 2026 11:00am</t>
         </is>
       </c>
       <c r="L208" s="1" t="n">
-        <v>45987.45833333334</v>
+        <v>46043.45833333334</v>
       </c>
       <c r="M208" t="inlineStr">
         <is>
-          <t>£250,000</t>
+          <t>£600,000</t>
         </is>
       </c>
       <c r="N208" s="1" t="n">
-        <v>45938</v>
+        <v>45931</v>
       </c>
     </row>
     <row r="209">
@@ -12654,21 +12816,21 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>ATI Programme strategic batch EoI – October 2025</t>
+          <t>CAM Pathfinder: Feasibility studies 2</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2317/overview/c946fbde-725e-4f85-bb3f-3219576c4a01</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2307/overview/8eec43e7-96a5-49d1-97e1-3400321160f9</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>2025-10-14 08:17</t>
+          <t>2025-10-10 08:18</t>
         </is>
       </c>
       <c r="E209" s="1" t="n">
-        <v>45944.34513888889</v>
+        <v>45940.34583333333</v>
       </c>
       <c r="F209" t="b">
         <v>1</v>
@@ -12681,13 +12843,17 @@
       <c r="J209" t="inlineStr"/>
       <c r="K209" t="inlineStr">
         <is>
-          <t>Wednesday 22 October 2025 11:00am</t>
+          <t>Wednesday 26 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L209" s="1" t="n">
-        <v>45952.45833333334</v>
-      </c>
-      <c r="M209" t="inlineStr"/>
+        <v>45987.45833333334</v>
+      </c>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>£250,000</t>
+        </is>
+      </c>
       <c r="N209" s="1" t="n">
         <v>45938</v>
       </c>
@@ -12700,21 +12866,21 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>CAM Pathfinder: Enable</t>
+          <t>ATI Programme strategic batch EoI – October 2025</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2318/overview/39cd0e04-6f9c-40da-b0be-8eaae7f1603d</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2317/overview/c946fbde-725e-4f85-bb3f-3219576c4a01</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>2025-10-15 08:19</t>
+          <t>2025-10-14 08:17</t>
         </is>
       </c>
       <c r="E210" s="1" t="n">
-        <v>45945.34652777778</v>
+        <v>45944.34513888889</v>
       </c>
       <c r="F210" t="b">
         <v>1</v>
@@ -12727,19 +12893,15 @@
       <c r="J210" t="inlineStr"/>
       <c r="K210" t="inlineStr">
         <is>
-          <t>Wednesday 17 December 2025 11:00am</t>
+          <t>Wednesday 22 October 2025 11:00am</t>
         </is>
       </c>
       <c r="L210" s="1" t="n">
-        <v>46008.45833333334</v>
-      </c>
-      <c r="M210" t="inlineStr">
-        <is>
-          <t>£4.0 million</t>
-        </is>
-      </c>
+        <v>45952.45833333334</v>
+      </c>
+      <c r="M210" t="inlineStr"/>
       <c r="N210" s="1" t="n">
-        <v>45945</v>
+        <v>45938</v>
       </c>
     </row>
     <row r="211">
@@ -12750,12 +12912,12 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>CAM Pathfinder: Demonstrate</t>
+          <t>CAM Pathfinder: Enable</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2315/overview/f02885bb-e043-4a60-8d0c-22242bd77fa9</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2318/overview/39cd0e04-6f9c-40da-b0be-8eaae7f1603d</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
@@ -12785,7 +12947,7 @@
       </c>
       <c r="M211" t="inlineStr">
         <is>
-          <t>£2.0 million</t>
+          <t>£4.0 million</t>
         </is>
       </c>
       <c r="N211" s="1" t="n">
@@ -12800,21 +12962,21 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Launchpad: life and health sciences, Northern Ireland – Rd3 MFA</t>
+          <t>CAM Pathfinder: Demonstrate</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2305/overview/fe565f48-36a8-4d8b-8515-e89d750f259c</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2315/overview/f02885bb-e043-4a60-8d0c-22242bd77fa9</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>2025-10-16 08:19</t>
+          <t>2025-10-15 08:19</t>
         </is>
       </c>
       <c r="E212" s="1" t="n">
-        <v>45946.34652777778</v>
+        <v>45945.34652777778</v>
       </c>
       <c r="F212" t="b">
         <v>1</v>
@@ -12827,15 +12989,15 @@
       <c r="J212" t="inlineStr"/>
       <c r="K212" t="inlineStr">
         <is>
-          <t>Wednesday 26 November 2025 11:00am</t>
+          <t>Wednesday 17 December 2025 11:00am</t>
         </is>
       </c>
       <c r="L212" s="1" t="n">
-        <v>45987.45833333334</v>
+        <v>46008.45833333334</v>
       </c>
       <c r="M212" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£2.0 million</t>
         </is>
       </c>
       <c r="N212" s="1" t="n">
@@ -12850,21 +13012,21 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>ADOPT Facilitator Support Grant: Round 5</t>
+          <t>Launchpad: life and health sciences, Northern Ireland – Rd3 MFA</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2299/overview/0a26e49f-fa03-4096-aa8b-3eb39b68f20d</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2305/overview/fe565f48-36a8-4d8b-8515-e89d750f259c</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>2025-10-17 08:19</t>
+          <t>2025-10-16 08:19</t>
         </is>
       </c>
       <c r="E213" s="1" t="n">
-        <v>45947.34652777778</v>
+        <v>45946.34652777778</v>
       </c>
       <c r="F213" t="b">
         <v>1</v>
@@ -12885,7 +13047,7 @@
       </c>
       <c r="M213" t="inlineStr">
         <is>
-          <t>£2,500</t>
+          <t>£100,000</t>
         </is>
       </c>
       <c r="N213" s="1" t="n">
@@ -12900,21 +13062,21 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Battery Innovation Feasibility Studies Round 1</t>
+          <t>ADOPT Facilitator Support Grant: Round 5</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2313/overview/508ab35f-0e07-4e84-8e31-bbbcb619bc9e</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2299/overview/0a26e49f-fa03-4096-aa8b-3eb39b68f20d</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>2025-10-18 08:16</t>
+          <t>2025-10-17 08:19</t>
         </is>
       </c>
       <c r="E214" s="1" t="n">
-        <v>45948.34444444445</v>
+        <v>45947.34652777778</v>
       </c>
       <c r="F214" t="b">
         <v>1</v>
@@ -12927,15 +13089,15 @@
       <c r="J214" t="inlineStr"/>
       <c r="K214" t="inlineStr">
         <is>
-          <t>Wednesday 17 December 2025 11:00am</t>
+          <t>Wednesday 26 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L214" s="1" t="n">
-        <v>46008.45833333334</v>
+        <v>45987.45833333334</v>
       </c>
       <c r="M214" t="inlineStr">
         <is>
-          <t>£500,000</t>
+          <t>£2,500</t>
         </is>
       </c>
       <c r="N214" s="1" t="n">
@@ -12950,12 +13112,12 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Battery Innovation Concept Development Round 1</t>
+          <t>Battery Innovation Feasibility Studies Round 1</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2314/overview/4d1e65d7-b380-41b7-8dcf-b25cd26b9ab5</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2313/overview/508ab35f-0e07-4e84-8e31-bbbcb619bc9e</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
@@ -12985,7 +13147,7 @@
       </c>
       <c r="M215" t="inlineStr">
         <is>
-          <t>£4.0 million</t>
+          <t>£500,000</t>
         </is>
       </c>
       <c r="N215" s="1" t="n">
@@ -13000,21 +13162,21 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>The Agentic AI Pioneers Prize</t>
+          <t>Battery Innovation Concept Development Round 1</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2316/overview/fa0eeab0-3021-4cbc-8975-5bd45a7d642a</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2314/overview/4d1e65d7-b380-41b7-8dcf-b25cd26b9ab5</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>2025-10-21 08:20</t>
+          <t>2025-10-18 08:16</t>
         </is>
       </c>
       <c r="E216" s="1" t="n">
-        <v>45951.34722222222</v>
+        <v>45948.34444444445</v>
       </c>
       <c r="F216" t="b">
         <v>1</v>
@@ -13027,13 +13189,17 @@
       <c r="J216" t="inlineStr"/>
       <c r="K216" t="inlineStr">
         <is>
-          <t>Wednesday 19 November 2025 11:00am</t>
+          <t>Wednesday 17 December 2025 11:00am</t>
         </is>
       </c>
       <c r="L216" s="1" t="n">
-        <v>45980.45833333334</v>
-      </c>
-      <c r="M216" t="inlineStr"/>
+        <v>46008.45833333334</v>
+      </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>£4.0 million</t>
+        </is>
+      </c>
       <c r="N216" s="1" t="n">
         <v>45945</v>
       </c>
@@ -13046,21 +13212,21 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>MSI: SME resource and energy efficiency – industrial research</t>
+          <t>The Agentic AI Pioneers Prize</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2328/overview/79cb058a-71b3-459a-93c2-8c96ecf7f18a</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2316/overview/fa0eeab0-3021-4cbc-8975-5bd45a7d642a</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>2025-10-22 08:21</t>
+          <t>2025-10-21 08:20</t>
         </is>
       </c>
       <c r="E217" s="1" t="n">
-        <v>45952.34791666667</v>
+        <v>45951.34722222222</v>
       </c>
       <c r="F217" t="b">
         <v>1</v>
@@ -13073,19 +13239,15 @@
       <c r="J217" t="inlineStr"/>
       <c r="K217" t="inlineStr">
         <is>
-          <t>Wednesday 10 December 2025 11:00am</t>
+          <t>Wednesday 19 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L217" s="1" t="n">
-        <v>46001.45833333334</v>
-      </c>
-      <c r="M217" t="inlineStr">
-        <is>
-          <t>£1.0 million</t>
-        </is>
-      </c>
+        <v>45980.45833333334</v>
+      </c>
+      <c r="M217" t="inlineStr"/>
       <c r="N217" s="1" t="n">
-        <v>45952</v>
+        <v>45945</v>
       </c>
     </row>
     <row r="218">
@@ -13096,12 +13258,12 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>MSI: SME resource and energy   efficiency – feasibility studies</t>
+          <t>MSI: SME resource and energy efficiency – industrial research</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2327/overview/bd7d1a37-69dc-4d09-8615-2bae4bcf3666</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2328/overview/79cb058a-71b3-459a-93c2-8c96ecf7f18a</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
@@ -13131,7 +13293,7 @@
       </c>
       <c r="M218" t="inlineStr">
         <is>
-          <t>£150,000</t>
+          <t>£1.0 million</t>
         </is>
       </c>
       <c r="N218" s="1" t="n">
@@ -13146,21 +13308,21 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Full ADOPT Grant Round 4</t>
+          <t>MSI: SME resource and energy   efficiency – feasibility studies</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2298/overview/71fd7055-502d-4f85-9127-749156a80fe6</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2327/overview/bd7d1a37-69dc-4d09-8615-2bae4bcf3666</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>2025-10-23 08:19</t>
+          <t>2025-10-22 08:21</t>
         </is>
       </c>
       <c r="E219" s="1" t="n">
-        <v>45953.34652777778</v>
+        <v>45952.34791666667</v>
       </c>
       <c r="F219" t="b">
         <v>1</v>
@@ -13181,7 +13343,7 @@
       </c>
       <c r="M219" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£150,000</t>
         </is>
       </c>
       <c r="N219" s="1" t="n">
@@ -13196,21 +13358,21 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Innovate UK Innovation Loans Round 24</t>
+          <t>Full ADOPT Grant Round 4</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2322/overview/1b933876-5f58-4dec-85ab-68b8c2722211</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2298/overview/71fd7055-502d-4f85-9127-749156a80fe6</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>2025-10-24 08:19</t>
+          <t>2025-10-23 08:19</t>
         </is>
       </c>
       <c r="E220" s="1" t="n">
-        <v>45954.34652777778</v>
+        <v>45953.34652777778</v>
       </c>
       <c r="F220" t="b">
         <v>1</v>
@@ -13223,15 +13385,15 @@
       <c r="J220" t="inlineStr"/>
       <c r="K220" t="inlineStr">
         <is>
-          <t>Wednesday 7 January 2026 11:00am</t>
+          <t>Wednesday 10 December 2025 11:00am</t>
         </is>
       </c>
       <c r="L220" s="1" t="n">
-        <v>46029.45833333334</v>
+        <v>46001.45833333334</v>
       </c>
       <c r="M220" t="inlineStr">
         <is>
-          <t>£5.0 million</t>
+          <t>£100,000</t>
         </is>
       </c>
       <c r="N220" s="1" t="n">
@@ -13246,21 +13408,21 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Knowledge Transfer Partnership (KTP): 2025 – 2026 Round 4</t>
+          <t>Innovate UK Innovation Loans Round 24</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2290/overview/8dd45f5c-3f38-4e38-b733-42b6cf601292</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2322/overview/1b933876-5f58-4dec-85ab-68b8c2722211</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>2025-10-25 08:16</t>
+          <t>2025-10-24 08:19</t>
         </is>
       </c>
       <c r="E221" s="1" t="n">
-        <v>45955.34444444445</v>
+        <v>45954.34652777778</v>
       </c>
       <c r="F221" t="b">
         <v>1</v>
@@ -13273,15 +13435,15 @@
       <c r="J221" t="inlineStr"/>
       <c r="K221" t="inlineStr">
         <is>
-          <t>Wednesday 26 November 2025 11:00am</t>
+          <t>Wednesday 7 January 2026 11:00am</t>
         </is>
       </c>
       <c r="L221" s="1" t="n">
-        <v>45987.45833333334</v>
+        <v>46029.45833333334</v>
       </c>
       <c r="M221" t="inlineStr">
         <is>
-          <t>£8,500</t>
+          <t>£5.0 million</t>
         </is>
       </c>
       <c r="N221" s="1" t="n">
@@ -13296,21 +13458,21 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>National Materials Innovation Programme: Feasibility Studies</t>
+          <t>Knowledge Transfer Partnership (KTP): 2025 – 2026 Round 4</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2326/overview/ca8aab61-a03b-431f-94a8-5c9b008495d5</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2290/overview/8dd45f5c-3f38-4e38-b733-42b6cf601292</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>2025-10-31 08:18</t>
+          <t>2025-10-25 08:16</t>
         </is>
       </c>
       <c r="E222" s="1" t="n">
-        <v>45961.34583333333</v>
+        <v>45955.34444444445</v>
       </c>
       <c r="F222" t="b">
         <v>1</v>
@@ -13323,19 +13485,19 @@
       <c r="J222" t="inlineStr"/>
       <c r="K222" t="inlineStr">
         <is>
-          <t>Wednesday 17 December 2025 11:00am</t>
+          <t>Wednesday 26 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L222" s="1" t="n">
-        <v>46008.45833333334</v>
+        <v>45987.45833333334</v>
       </c>
       <c r="M222" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£8,500</t>
         </is>
       </c>
       <c r="N222" s="1" t="n">
-        <v>45959</v>
+        <v>45952</v>
       </c>
     </row>
     <row r="223">
@@ -13346,21 +13508,21 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>UK-Canada Quantum Communications and Networking Demonstrator</t>
+          <t>National Materials Innovation Programme: Feasibility Studies</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2335/overview/64e26f1b-8564-4539-b3ca-1b15ebf4f94a</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2326/overview/ca8aab61-a03b-431f-94a8-5c9b008495d5</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>2025-11-04 08:20</t>
+          <t>2025-10-31 08:18</t>
         </is>
       </c>
       <c r="E223" s="1" t="n">
-        <v>45965.34722222222</v>
+        <v>45961.34583333333</v>
       </c>
       <c r="F223" t="b">
         <v>1</v>
@@ -13373,15 +13535,15 @@
       <c r="J223" t="inlineStr"/>
       <c r="K223" t="inlineStr">
         <is>
-          <t>Wednesday 26 November 2025 11:00am</t>
+          <t>Wednesday 17 December 2025 11:00am</t>
         </is>
       </c>
       <c r="L223" s="1" t="n">
-        <v>45987.45833333334</v>
+        <v>46008.45833333334</v>
       </c>
       <c r="M223" t="inlineStr">
         <is>
-          <t>£3.4 million</t>
+          <t>£100,000</t>
         </is>
       </c>
       <c r="N223" s="1" t="n">
@@ -13396,12 +13558,12 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Increasing EV charging capacity on the strategic road network</t>
+          <t>UK-Canada Quantum Communications and Networking Demonstrator</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2304/overview/9ea6670e-83fd-43f9-972f-e0eff8fe77a8</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2335/overview/64e26f1b-8564-4539-b3ca-1b15ebf4f94a</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
@@ -13423,15 +13585,15 @@
       <c r="J224" t="inlineStr"/>
       <c r="K224" t="inlineStr">
         <is>
-          <t>Wednesday 25 March 2026 11:00am</t>
+          <t>Wednesday 26 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L224" s="1" t="n">
-        <v>46106.45833333334</v>
+        <v>45987.45833333334</v>
       </c>
       <c r="M224" t="inlineStr">
         <is>
-          <t>£3.0 million</t>
+          <t>£3.4 million</t>
         </is>
       </c>
       <c r="N224" s="1" t="n">
@@ -13446,21 +13608,21 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Biomedical Catalyst 2025: Industry led R&amp;D small projects</t>
+          <t>Increasing EV charging capacity on the strategic road network</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2333/overview/f5431c75-e2e1-48f4-bc8e-62d52121cb6f</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2304/overview/9ea6670e-83fd-43f9-972f-e0eff8fe77a8</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>2025-11-05 08:19</t>
+          <t>2025-11-04 08:20</t>
         </is>
       </c>
       <c r="E225" s="1" t="n">
-        <v>45966.34652777778</v>
+        <v>45965.34722222222</v>
       </c>
       <c r="F225" t="b">
         <v>1</v>
@@ -13473,19 +13635,19 @@
       <c r="J225" t="inlineStr"/>
       <c r="K225" t="inlineStr">
         <is>
-          <t>Wednesday 10 December 2025 11:00am</t>
+          <t>Wednesday 25 March 2026 11:00am</t>
         </is>
       </c>
       <c r="L225" s="1" t="n">
-        <v>46001.45833333334</v>
+        <v>46106.45833333334</v>
       </c>
       <c r="M225" t="inlineStr">
         <is>
-          <t>£1.0 million</t>
+          <t>£3.0 million</t>
         </is>
       </c>
       <c r="N225" s="1" t="n">
-        <v>45966</v>
+        <v>45959</v>
       </c>
     </row>
     <row r="226">
@@ -13496,12 +13658,12 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Biomedical Catalyst 2025: Industry led R&amp;D large projects</t>
+          <t>Biomedical Catalyst 2025: Industry led R&amp;D small projects</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2332/overview/bf6bd8c3-e550-478d-b374-a3cb0fb4d3d3</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2333/overview/f5431c75-e2e1-48f4-bc8e-62d52121cb6f</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
@@ -13531,7 +13693,7 @@
       </c>
       <c r="M226" t="inlineStr">
         <is>
-          <t>£4.0 million</t>
+          <t>£1.0 million</t>
         </is>
       </c>
       <c r="N226" s="1" t="n">
@@ -13546,12 +13708,12 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>ATI Programme strategic batch EoI – November 2025</t>
+          <t>Biomedical Catalyst 2025: Industry led R&amp;D large projects</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2334/overview/4af06b80-2953-4cb3-8cc0-987ec5a2f322</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2332/overview/bf6bd8c3-e550-478d-b374-a3cb0fb4d3d3</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
@@ -13573,13 +13735,17 @@
       <c r="J227" t="inlineStr"/>
       <c r="K227" t="inlineStr">
         <is>
-          <t>Wednesday 19 November 2025 11:00am</t>
+          <t>Wednesday 10 December 2025 11:00am</t>
         </is>
       </c>
       <c r="L227" s="1" t="n">
-        <v>45980.45833333334</v>
-      </c>
-      <c r="M227" t="inlineStr"/>
+        <v>46001.45833333334</v>
+      </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>£4.0 million</t>
+        </is>
+      </c>
       <c r="N227" s="1" t="n">
         <v>45966</v>
       </c>
@@ -13592,21 +13758,21 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>DRIVE35 Scale-up: Feasibility Studies 2</t>
+          <t>ATI Programme strategic batch EoI – November 2025</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2341/overview/4b0efce9-75b8-4e84-97c0-fc6277396586</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2334/overview/4af06b80-2953-4cb3-8cc0-987ec5a2f322</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>2025-11-11 08:19</t>
+          <t>2025-11-05 08:19</t>
         </is>
       </c>
       <c r="E228" s="1" t="n">
-        <v>45972.34652777778</v>
+        <v>45966.34652777778</v>
       </c>
       <c r="F228" t="b">
         <v>1</v>
@@ -13619,17 +13785,13 @@
       <c r="J228" t="inlineStr"/>
       <c r="K228" t="inlineStr">
         <is>
-          <t>Wednesday 17 December 2025 11:00am</t>
+          <t>Wednesday 19 November 2025 11:00am</t>
         </is>
       </c>
       <c r="L228" s="1" t="n">
-        <v>46008.45833333334</v>
-      </c>
-      <c r="M228" t="inlineStr">
-        <is>
-          <t>£750,000</t>
-        </is>
-      </c>
+        <v>45980.45833333334</v>
+      </c>
+      <c r="M228" t="inlineStr"/>
       <c r="N228" s="1" t="n">
         <v>45966</v>
       </c>
@@ -13642,21 +13804,21 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Women in Innovation Awards 2025/26</t>
+          <t>DRIVE35 Scale-up: Feasibility Studies 2</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2337/overview/3750b1cd-2080-4a1c-82c0-003fbaafdd2d</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2341/overview/4b0efce9-75b8-4e84-97c0-fc6277396586</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>2025-11-27 13:23</t>
+          <t>2025-11-11 08:19</t>
         </is>
       </c>
       <c r="E229" s="1" t="n">
-        <v>45988.55763888889</v>
+        <v>45972.34652777778</v>
       </c>
       <c r="F229" t="b">
         <v>1</v>
@@ -13669,19 +13831,19 @@
       <c r="J229" t="inlineStr"/>
       <c r="K229" t="inlineStr">
         <is>
-          <t>Wednesday 4 February 2026 11:00am</t>
+          <t>Wednesday 17 December 2025 11:00am</t>
         </is>
       </c>
       <c r="L229" s="1" t="n">
-        <v>46057.45833333334</v>
+        <v>46008.45833333334</v>
       </c>
       <c r="M229" t="inlineStr">
         <is>
-          <t>£75,000</t>
+          <t>£750,000</t>
         </is>
       </c>
       <c r="N229" s="1" t="n">
-        <v>45987</v>
+        <v>45966</v>
       </c>
     </row>
     <row r="230">
@@ -13692,21 +13854,21 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Knowledge Transfer Partnership (KTP): 2025 – 2026 Round 5</t>
+          <t>Women in Innovation Awards 2025/26</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2354/overview/c7008321-f651-45c5-a409-c3215231fbb4</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2337/overview/3750b1cd-2080-4a1c-82c0-003fbaafdd2d</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>2025-12-02 08:22</t>
+          <t>2025-11-27 13:23</t>
         </is>
       </c>
       <c r="E230" s="1" t="n">
-        <v>45993.34861111111</v>
+        <v>45988.55763888889</v>
       </c>
       <c r="F230" t="b">
         <v>1</v>
@@ -13727,7 +13889,7 @@
       </c>
       <c r="M230" t="inlineStr">
         <is>
-          <t>£8,500</t>
+          <t>£75,000</t>
         </is>
       </c>
       <c r="N230" s="1" t="n">
@@ -13742,21 +13904,21 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Innovate UK Growth Catalyst – Investor Partnerships Round 2</t>
+          <t>Knowledge Transfer Partnership (KTP): 2025 – 2026 Round 5</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2360/overview/37d8f6e1-5600-4e9e-bbfc-11bc320f8808</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2354/overview/c7008321-f651-45c5-a409-c3215231fbb4</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>2025-12-11 08:22</t>
+          <t>2025-12-02 08:22</t>
         </is>
       </c>
       <c r="E231" s="1" t="n">
-        <v>46002.34861111111</v>
+        <v>45993.34861111111</v>
       </c>
       <c r="F231" t="b">
         <v>1</v>
@@ -13769,19 +13931,19 @@
       <c r="J231" t="inlineStr"/>
       <c r="K231" t="inlineStr">
         <is>
-          <t>Tuesday 3 February 2026 11:00am</t>
+          <t>Wednesday 4 February 2026 11:00am</t>
         </is>
       </c>
       <c r="L231" s="1" t="n">
-        <v>46056.45833333334</v>
+        <v>46057.45833333334</v>
       </c>
       <c r="M231" t="inlineStr">
         <is>
-          <t>£2.0 million</t>
+          <t>£8,500</t>
         </is>
       </c>
       <c r="N231" s="1" t="n">
-        <v>46001</v>
+        <v>45987</v>
       </c>
     </row>
     <row r="232">
@@ -13792,21 +13954,21 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Full ADOPT Grant: Round 5</t>
+          <t>Innovate UK Growth Catalyst – Investor Partnerships Round 2</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2358/overview/f93f32c2-dd04-474d-bc35-a8af1ecac1a9</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2360/overview/37d8f6e1-5600-4e9e-bbfc-11bc320f8808</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>2025-12-12 08:22</t>
+          <t>2025-12-11 08:22</t>
         </is>
       </c>
       <c r="E232" s="1" t="n">
-        <v>46003.34861111111</v>
+        <v>46002.34861111111</v>
       </c>
       <c r="F232" t="b">
         <v>1</v>
@@ -13819,15 +13981,15 @@
       <c r="J232" t="inlineStr"/>
       <c r="K232" t="inlineStr">
         <is>
-          <t>Wednesday 4 February 2026 11:00am</t>
+          <t>Tuesday 3 February 2026 11:00am</t>
         </is>
       </c>
       <c r="L232" s="1" t="n">
-        <v>46057.45833333334</v>
+        <v>46056.45833333334</v>
       </c>
       <c r="M232" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£2.0 million</t>
         </is>
       </c>
       <c r="N232" s="1" t="n">
@@ -13842,21 +14004,21 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>ADOPT Facilitator Support Grant: Round 6</t>
+          <t>Full ADOPT Grant: Round 5</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2371/overview/471bfe91-9f9c-4086-a28a-15296f1957e2</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2358/overview/f93f32c2-dd04-474d-bc35-a8af1ecac1a9</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>2025-12-18 08:21</t>
+          <t>2025-12-12 08:22</t>
         </is>
       </c>
       <c r="E233" s="1" t="n">
-        <v>46009.34791666667</v>
+        <v>46003.34861111111</v>
       </c>
       <c r="F233" t="b">
         <v>1</v>
@@ -13869,19 +14031,19 @@
       <c r="J233" t="inlineStr"/>
       <c r="K233" t="inlineStr">
         <is>
-          <t>Wednesday 25 February 2026 11:00am</t>
+          <t>Wednesday 4 February 2026 11:00am</t>
         </is>
       </c>
       <c r="L233" s="1" t="n">
-        <v>46078.45833333334</v>
+        <v>46057.45833333334</v>
       </c>
       <c r="M233" t="inlineStr">
         <is>
-          <t>£2,500</t>
+          <t>£100,000</t>
         </is>
       </c>
       <c r="N233" s="1" t="n">
-        <v>46008</v>
+        <v>46001</v>
       </c>
     </row>
     <row r="234">
@@ -13892,12 +14054,12 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Commercialising Knowledge Assets Fund (CKAF) Spring</t>
+          <t>ADOPT Facilitator Support Grant: Round 6</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2369/overview/abf7d399-81b9-4f33-b592-51825a288c37</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2371/overview/471bfe91-9f9c-4086-a28a-15296f1957e2</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
@@ -13919,15 +14081,15 @@
       <c r="J234" t="inlineStr"/>
       <c r="K234" t="inlineStr">
         <is>
-          <t>Thursday 7 May 2026 11:00am</t>
+          <t>Wednesday 25 February 2026 11:00am</t>
         </is>
       </c>
       <c r="L234" s="1" t="n">
-        <v>46149.45833333334</v>
+        <v>46078.45833333334</v>
       </c>
       <c r="M234" t="inlineStr">
         <is>
-          <t>£250,000</t>
+          <t>£2,500</t>
         </is>
       </c>
       <c r="N234" s="1" t="n">
@@ -13942,21 +14104,21 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Energy catalyst round 11 – mid stage</t>
+          <t>Commercialising Knowledge Assets Fund (CKAF) Spring</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2363/overview/9f759af1-3732-4d15-995d-053e28025d22</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2369/overview/abf7d399-81b9-4f33-b592-51825a288c37</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>2026-01-06 08:22</t>
+          <t>2025-12-18 08:21</t>
         </is>
       </c>
       <c r="E235" s="1" t="n">
-        <v>46028.34861111111</v>
+        <v>46009.34791666667</v>
       </c>
       <c r="F235" t="b">
         <v>1</v>
@@ -13969,19 +14131,19 @@
       <c r="J235" t="inlineStr"/>
       <c r="K235" t="inlineStr">
         <is>
-          <t>Wednesday 25 March 2026 11:00am</t>
+          <t>Thursday 7 May 2026 11:00am</t>
         </is>
       </c>
       <c r="L235" s="1" t="n">
-        <v>46106.45833333334</v>
+        <v>46149.45833333334</v>
       </c>
       <c r="M235" t="inlineStr">
         <is>
-          <t>£1.5 million</t>
+          <t>£250,000</t>
         </is>
       </c>
       <c r="N235" s="1" t="n">
-        <v>46022</v>
+        <v>46008</v>
       </c>
     </row>
     <row r="236">
@@ -13992,12 +14154,12 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Energy catalyst round 11 – late stage</t>
+          <t>Energy catalyst round 11 – mid stage</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2364/overview/b9d4dedf-d22a-41d1-9ca2-6c5a279519be</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2363/overview/9f759af1-3732-4d15-995d-053e28025d22</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
@@ -14027,7 +14189,7 @@
       </c>
       <c r="M236" t="inlineStr">
         <is>
-          <t>£5.0 million</t>
+          <t>£1.5 million</t>
         </is>
       </c>
       <c r="N236" s="1" t="n">
@@ -14042,12 +14204,12 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Energy catalyst round 11 – early stage</t>
+          <t>Energy catalyst round 11 – late stage</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2362/overview/640b2f4e-8571-4aef-9e2a-67e35db3db77</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2364/overview/b9d4dedf-d22a-41d1-9ca2-6c5a279519be</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -14077,7 +14239,7 @@
       </c>
       <c r="M237" t="inlineStr">
         <is>
-          <t>£300,000</t>
+          <t>£5.0 million</t>
         </is>
       </c>
       <c r="N237" s="1" t="n">
@@ -14092,12 +14254,12 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>DRIVE35 Innovation Fund: Demonstrate 2</t>
+          <t>Energy catalyst round 11 – early stage</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2351/overview/349c38f5-5ed2-4cf4-a324-bda2d6cd1e67</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2362/overview/640b2f4e-8571-4aef-9e2a-67e35db3db77</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -14119,15 +14281,15 @@
       <c r="J238" t="inlineStr"/>
       <c r="K238" t="inlineStr">
         <is>
-          <t>Wednesday 11 March 2026 11:00am</t>
+          <t>Wednesday 25 March 2026 11:00am</t>
         </is>
       </c>
       <c r="L238" s="1" t="n">
-        <v>46092.45833333334</v>
+        <v>46106.45833333334</v>
       </c>
       <c r="M238" t="inlineStr">
         <is>
-          <t>£1.5 million</t>
+          <t>£300,000</t>
         </is>
       </c>
       <c r="N238" s="1" t="n">
@@ -14142,12 +14304,12 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>DRIVE35 Innovation Fund: Collaborate 2</t>
+          <t>DRIVE35 Innovation Fund: Demonstrate 2</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2350/overview/dbd41be3-14ea-4c83-8774-eb28a8703d57</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2351/overview/349c38f5-5ed2-4cf4-a324-bda2d6cd1e67</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
@@ -14169,15 +14331,15 @@
       <c r="J239" t="inlineStr"/>
       <c r="K239" t="inlineStr">
         <is>
-          <t>Wednesday 18 March 2026 11:00am</t>
+          <t>Wednesday 11 March 2026 11:00am</t>
         </is>
       </c>
       <c r="L239" s="1" t="n">
-        <v>46099.45833333334</v>
+        <v>46092.45833333334</v>
       </c>
       <c r="M239" t="inlineStr">
         <is>
-          <t>£25.0 million</t>
+          <t>£1.5 million</t>
         </is>
       </c>
       <c r="N239" s="1" t="n">
@@ -14192,21 +14354,21 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Innovate UK Innovation Loans Round 25</t>
+          <t>DRIVE35 Innovation Fund: Collaborate 2</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2373/overview/609dc5dd-d3e8-4f51-af3a-3eb1b3314710</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2350/overview/dbd41be3-14ea-4c83-8774-eb28a8703d57</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>2026-01-08 08:22</t>
+          <t>2026-01-06 08:22</t>
         </is>
       </c>
       <c r="E240" s="1" t="n">
-        <v>46030.34861111111</v>
+        <v>46028.34861111111</v>
       </c>
       <c r="F240" t="b">
         <v>1</v>
@@ -14219,19 +14381,19 @@
       <c r="J240" t="inlineStr"/>
       <c r="K240" t="inlineStr">
         <is>
-          <t>Wednesday 4 March 2026 11:00am</t>
+          <t>Wednesday 18 March 2026 11:00am</t>
         </is>
       </c>
       <c r="L240" s="1" t="n">
-        <v>46085.45833333334</v>
+        <v>46099.45833333334</v>
       </c>
       <c r="M240" t="inlineStr">
         <is>
-          <t>£5.0 million</t>
+          <t>£25.0 million</t>
         </is>
       </c>
       <c r="N240" s="1" t="n">
-        <v>46029</v>
+        <v>46022</v>
       </c>
     </row>
     <row r="241">
@@ -14242,21 +14404,21 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Cyber Security Academic Startup Accelerator Programme Y10 Phase 1</t>
+          <t>Innovate UK Innovation Loans Round 25</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2376/overview/1b9b9265-ca4b-4f8c-a0c2-577cb8713642</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2373/overview/609dc5dd-d3e8-4f51-af3a-3eb1b3314710</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>2026-01-15 08:23</t>
+          <t>2026-01-08 08:22</t>
         </is>
       </c>
       <c r="E241" s="1" t="n">
-        <v>46037.34930555556</v>
+        <v>46030.34861111111</v>
       </c>
       <c r="F241" t="b">
         <v>1</v>
@@ -14269,19 +14431,19 @@
       <c r="J241" t="inlineStr"/>
       <c r="K241" t="inlineStr">
         <is>
-          <t>Wednesday 11 February 2026 11:00am</t>
+          <t>Wednesday 4 March 2026 11:00am</t>
         </is>
       </c>
       <c r="L241" s="1" t="n">
-        <v>46064.45833333334</v>
+        <v>46085.45833333334</v>
       </c>
       <c r="M241" t="inlineStr">
         <is>
-          <t>£32,000</t>
+          <t>£5.0 million</t>
         </is>
       </c>
       <c r="N241" s="1" t="n">
-        <v>46036</v>
+        <v>46029</v>
       </c>
     </row>
     <row r="242">
@@ -14292,21 +14454,21 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Ofgem Strategic Innovation Fund Round 5 Discovery C5</t>
+          <t>Cyber Security Academic Startup Accelerator Programme Y10 Phase 1</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2346/overview/e172ee7c-3050-4d47-bf11-235cfe76c1e1</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2376/overview/1b9b9265-ca4b-4f8c-a0c2-577cb8713642</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>2026-01-20 08:24</t>
+          <t>2026-01-15 08:23</t>
         </is>
       </c>
       <c r="E242" s="1" t="n">
-        <v>46042.35</v>
+        <v>46037.34930555556</v>
       </c>
       <c r="F242" t="b">
         <v>1</v>
@@ -14319,15 +14481,15 @@
       <c r="J242" t="inlineStr"/>
       <c r="K242" t="inlineStr">
         <is>
-          <t>Wednesday 25 February 2026 11:00am</t>
+          <t>Wednesday 11 February 2026 11:00am</t>
         </is>
       </c>
       <c r="L242" s="1" t="n">
-        <v>46078.45833333334</v>
+        <v>46064.45833333334</v>
       </c>
       <c r="M242" t="inlineStr">
         <is>
-          <t>£150,000</t>
+          <t>£32,000</t>
         </is>
       </c>
       <c r="N242" s="1" t="n">
@@ -14342,21 +14504,21 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Advanced manufacturing supply chain innovation FS</t>
+          <t>Ofgem Strategic Innovation Fund Round 5 Discovery C5</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2384/overview/2ad8ce21-d3f6-48bf-b55a-5af2a892a1e0</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2346/overview/e172ee7c-3050-4d47-bf11-235cfe76c1e1</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>2026-01-26 12:10</t>
+          <t>2026-01-20 08:24</t>
         </is>
       </c>
       <c r="E243" s="1" t="n">
-        <v>46048.50694444445</v>
+        <v>46042.35</v>
       </c>
       <c r="F243" t="b">
         <v>1</v>
@@ -14369,19 +14531,19 @@
       <c r="J243" t="inlineStr"/>
       <c r="K243" t="inlineStr">
         <is>
-          <t>Wednesday 11 March 2026 11:00am</t>
+          <t>Wednesday 25 February 2026 11:00am</t>
         </is>
       </c>
       <c r="L243" s="1" t="n">
-        <v>46092.45833333334</v>
+        <v>46078.45833333334</v>
       </c>
       <c r="M243" t="inlineStr">
         <is>
-          <t>£100,000</t>
+          <t>£150,000</t>
         </is>
       </c>
       <c r="N243" s="1" t="n">
-        <v>46043</v>
+        <v>46036</v>
       </c>
     </row>
     <row r="244">
@@ -14392,21 +14554,21 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>TechLocal: Connecting Local Talent to Local Tech Jobs</t>
+          <t>Advanced manufacturing supply chain innovation FS</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2378/overview/ae120ce2-7b72-4cf2-8dde-f78b02d5996d</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2384/overview/2ad8ce21-d3f6-48bf-b55a-5af2a892a1e0</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>2026-01-28 10:24</t>
+          <t>2026-01-26 12:10</t>
         </is>
       </c>
       <c r="E244" s="1" t="n">
-        <v>46050.43333333333</v>
+        <v>46048.50694444445</v>
       </c>
       <c r="F244" t="b">
         <v>1</v>
@@ -14419,19 +14581,19 @@
       <c r="J244" t="inlineStr"/>
       <c r="K244" t="inlineStr">
         <is>
-          <t>Wednesday 18 March 2026 11:00am</t>
+          <t>Wednesday 11 March 2026 11:00am</t>
         </is>
       </c>
       <c r="L244" s="1" t="n">
-        <v>46099.45833333334</v>
+        <v>46092.45833333334</v>
       </c>
       <c r="M244" t="inlineStr">
         <is>
-          <t>£225,000</t>
+          <t>£100,000</t>
         </is>
       </c>
       <c r="N244" s="1" t="n">
-        <v>46050</v>
+        <v>46043</v>
       </c>
     </row>
     <row r="245">
@@ -14442,12 +14604,12 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>TechLocal AI Professional Degree and Traineeship Accelerator</t>
+          <t>TechLocal: Connecting Local Talent to Local Tech Jobs</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2375/overview/6431359e-eb5c-4f76-b49d-299948107fbd</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2378/overview/ae120ce2-7b72-4cf2-8dde-f78b02d5996d</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -14477,7 +14639,7 @@
       </c>
       <c r="M245" t="inlineStr">
         <is>
-          <t>£300,000</t>
+          <t>£225,000</t>
         </is>
       </c>
       <c r="N245" s="1" t="n">
@@ -14492,21 +14654,21 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Robotics Adoption Programme skills development</t>
+          <t>TechLocal AI Professional Degree and Traineeship Accelerator</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2387/overview/daca31c2-8395-4bc2-a5da-55eb1e432fa4</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2375/overview/6431359e-eb5c-4f76-b49d-299948107fbd</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>2026-02-02 10:39</t>
+          <t>2026-01-28 10:24</t>
         </is>
       </c>
       <c r="E246" s="1" t="n">
-        <v>46055.44375</v>
+        <v>46050.43333333333</v>
       </c>
       <c r="F246" t="b">
         <v>1</v>
@@ -14519,15 +14681,15 @@
       <c r="J246" t="inlineStr"/>
       <c r="K246" t="inlineStr">
         <is>
-          <t>Wednesday 25 March 2026 11:00am</t>
+          <t>Wednesday 18 March 2026 11:00am</t>
         </is>
       </c>
       <c r="L246" s="1" t="n">
-        <v>46106.45833333334</v>
+        <v>46099.45833333334</v>
       </c>
       <c r="M246" t="inlineStr">
         <is>
-          <t>£500,000</t>
+          <t>£300,000</t>
         </is>
       </c>
       <c r="N246" s="1" t="n">
@@ -14542,21 +14704,21 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Knowledge Transfer Partnership (KTP): 2026 – 2027 Round 1</t>
+          <t>Robotics Adoption Programme skills development</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2380/overview/3e170dd3-4458-4c7e-a096-e0ea50b88040</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2387/overview/daca31c2-8395-4bc2-a5da-55eb1e432fa4</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>2026-02-03 10:35</t>
+          <t>2026-02-02 10:39</t>
         </is>
       </c>
       <c r="E247" s="1" t="n">
-        <v>46056.44097222222</v>
+        <v>46055.44375</v>
       </c>
       <c r="F247" t="b">
         <v>1</v>
@@ -14569,15 +14731,15 @@
       <c r="J247" t="inlineStr"/>
       <c r="K247" t="inlineStr">
         <is>
-          <t>Wednesday 1 April 2026 11:00am</t>
+          <t>Wednesday 25 March 2026 11:00am</t>
         </is>
       </c>
       <c r="L247" s="1" t="n">
-        <v>46113.45833333334</v>
+        <v>46106.45833333334</v>
       </c>
       <c r="M247" t="inlineStr">
         <is>
-          <t>£8,500</t>
+          <t>£500,000</t>
         </is>
       </c>
       <c r="N247" s="1" t="n">
@@ -14592,12 +14754,12 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Biomedical Catalyst Accelerator Provider Pool EoI: late stage</t>
+          <t>Knowledge Transfer Partnership (KTP): 2026 – 2027 Round 1</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2389/overview/a7f7d874-8b6b-45d6-b1e1-1e88e11a1ea5</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2380/overview/3e170dd3-4458-4c7e-a096-e0ea50b88040</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -14619,13 +14781,17 @@
       <c r="J248" t="inlineStr"/>
       <c r="K248" t="inlineStr">
         <is>
-          <t>Wednesday 4 March 2026 11:00am</t>
+          <t>Wednesday 1 April 2026 11:00am</t>
         </is>
       </c>
       <c r="L248" s="1" t="n">
-        <v>46085.45833333334</v>
-      </c>
-      <c r="M248" t="inlineStr"/>
+        <v>46113.45833333334</v>
+      </c>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>£8,500</t>
+        </is>
+      </c>
       <c r="N248" s="1" t="n">
         <v>46050</v>
       </c>
@@ -14638,12 +14804,12 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Biomedical Catalyst Accelerator Provider Pool EoI: early stage</t>
+          <t>Biomedical Catalyst Accelerator Provider Pool EoI: late stage</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2388/overview/08b8ab63-085d-4d79-ae83-e8c1698cb327</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2389/overview/a7f7d874-8b6b-45d6-b1e1-1e88e11a1ea5</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
@@ -14684,21 +14850,21 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Full ADOPT Grant: Round 6</t>
+          <t>Biomedical Catalyst Accelerator Provider Pool EoI: early stage</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2385/overview/2343c344-807d-41a1-9551-05ac5420ba11</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2388/overview/08b8ab63-085d-4d79-ae83-e8c1698cb327</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>2026-02-09 10:53</t>
+          <t>2026-02-03 10:35</t>
         </is>
       </c>
       <c r="E250" s="1" t="n">
-        <v>46062.45347222222</v>
+        <v>46056.44097222222</v>
       </c>
       <c r="F250" t="b">
         <v>1</v>
@@ -14711,19 +14877,15 @@
       <c r="J250" t="inlineStr"/>
       <c r="K250" t="inlineStr">
         <is>
-          <t>Wednesday 8 April 2026 11:00am</t>
+          <t>Wednesday 4 March 2026 11:00am</t>
         </is>
       </c>
       <c r="L250" s="1" t="n">
-        <v>46120.45833333334</v>
-      </c>
-      <c r="M250" t="inlineStr">
-        <is>
-          <t>£100,000</t>
-        </is>
-      </c>
+        <v>46085.45833333334</v>
+      </c>
+      <c r="M250" t="inlineStr"/>
       <c r="N250" s="1" t="n">
-        <v>46057</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="251">
@@ -14734,21 +14896,21 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Zero Emission Flight Demonstrator Round 1</t>
+          <t>Full ADOPT Grant: Round 6</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2397/overview/752074ec-5f01-46d8-863f-596300a11651</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2385/overview/2343c344-807d-41a1-9551-05ac5420ba11</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>2026-02-12 10:40</t>
+          <t>2026-02-09 10:53</t>
         </is>
       </c>
       <c r="E251" s="1" t="n">
-        <v>46065.44444444445</v>
+        <v>46062.45347222222</v>
       </c>
       <c r="F251" t="b">
         <v>1</v>
@@ -14761,19 +14923,19 @@
       <c r="J251" t="inlineStr"/>
       <c r="K251" t="inlineStr">
         <is>
-          <t>Wednesday 1 April 2026 11:00am</t>
+          <t>Wednesday 8 April 2026 11:00am</t>
         </is>
       </c>
       <c r="L251" s="1" t="n">
-        <v>46113.45833333334</v>
+        <v>46120.45833333334</v>
       </c>
       <c r="M251" t="inlineStr">
         <is>
-          <t>£5.0 million</t>
+          <t>£100,000</t>
         </is>
       </c>
       <c r="N251" s="1" t="n">
-        <v>46064</v>
+        <v>46057</v>
       </c>
     </row>
     <row r="252">
@@ -14784,12 +14946,12 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Contracts for Innovation in drug and alcohol addiction healthcare</t>
+          <t>Zero Emission Flight Demonstrator Round 1</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2395/overview/3d49fbc4-6e09-4dd8-9ac8-8e5f88facd8d</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2397/overview/752074ec-5f01-46d8-863f-596300a11651</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -14811,15 +14973,15 @@
       <c r="J252" t="inlineStr"/>
       <c r="K252" t="inlineStr">
         <is>
-          <t>Wednesday 6 May 2026 11:00am</t>
+          <t>Wednesday 1 April 2026 11:00am</t>
         </is>
       </c>
       <c r="L252" s="1" t="n">
-        <v>46148.45833333334</v>
+        <v>46113.45833333334</v>
       </c>
       <c r="M252" t="inlineStr">
         <is>
-          <t>£1.5 million</t>
+          <t>£5.0 million</t>
         </is>
       </c>
       <c r="N252" s="1" t="n">
@@ -14834,12 +14996,12 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Advancing innovation in drug and alcohol addiction healthcare</t>
+          <t>Contracts for Innovation in drug and alcohol addiction healthcare</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2394/overview/33b56af8-353f-46ac-bb66-a0928731c0fc</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2395/overview/3d49fbc4-6e09-4dd8-9ac8-8e5f88facd8d</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -14869,7 +15031,7 @@
       </c>
       <c r="M253" t="inlineStr">
         <is>
-          <t>£10.0 million</t>
+          <t>£1.5 million</t>
         </is>
       </c>
       <c r="N253" s="1" t="n">
@@ -14884,21 +15046,21 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>UK-Germany Collaborative Innovation for Quantum Technologies 2026</t>
+          <t>Advancing innovation in drug and alcohol addiction healthcare</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2392/overview/b8b93732-6326-4aed-9af3-334e4cc5ecc0</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2394/overview/33b56af8-353f-46ac-bb66-a0928731c0fc</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>2026-02-13 10:35</t>
+          <t>2026-02-12 10:40</t>
         </is>
       </c>
       <c r="E254" s="1" t="n">
-        <v>46066.44097222222</v>
+        <v>46065.44444444445</v>
       </c>
       <c r="F254" t="b">
         <v>1</v>
@@ -14911,15 +15073,15 @@
       <c r="J254" t="inlineStr"/>
       <c r="K254" t="inlineStr">
         <is>
-          <t>Wednesday 15 April 2026 11:00am</t>
+          <t>Wednesday 6 May 2026 11:00am</t>
         </is>
       </c>
       <c r="L254" s="1" t="n">
-        <v>46127.45833333334</v>
+        <v>46148.45833333334</v>
       </c>
       <c r="M254" t="inlineStr">
         <is>
-          <t>£1.0 million</t>
+          <t>£10.0 million</t>
         </is>
       </c>
       <c r="N254" s="1" t="n">
@@ -14934,21 +15096,21 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Contracts for Innovation: industrial human relevant drug models</t>
+          <t>UK-Germany Collaborative Innovation for Quantum Technologies 2026</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2396/overview/d55398bb-ff62-43b9-9ee1-bf3fa4b95c5c</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2392/overview/b8b93732-6326-4aed-9af3-334e4cc5ecc0</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>2026-02-17 10:40</t>
+          <t>2026-02-13 10:35</t>
         </is>
       </c>
       <c r="E255" s="1" t="n">
-        <v>46070.44444444445</v>
+        <v>46066.44097222222</v>
       </c>
       <c r="F255" t="b">
         <v>1</v>
@@ -14969,7 +15131,7 @@
       </c>
       <c r="M255" t="inlineStr">
         <is>
-          <t>£200,000</t>
+          <t>£1.0 million</t>
         </is>
       </c>
       <c r="N255" s="1" t="n">
@@ -14984,21 +15146,21 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Semiconductors and components for smart electronic platforms</t>
+          <t>Contracts for Innovation: industrial human relevant drug models</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2403/overview/4b54c133-c9b2-4572-9cca-2a7a4f69e5b8</t>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2396/overview/d55398bb-ff62-43b9-9ee1-bf3fa4b95c5c</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>2026-02-20 10:32</t>
+          <t>2026-02-17 10:40</t>
         </is>
       </c>
       <c r="E256" s="1" t="n">
-        <v>46073.43888888889</v>
+        <v>46070.44444444445</v>
       </c>
       <c r="F256" t="b">
         <v>1</v>
@@ -15011,18 +15173,168 @@
       <c r="J256" t="inlineStr"/>
       <c r="K256" t="inlineStr">
         <is>
+          <t>Wednesday 15 April 2026 11:00am</t>
+        </is>
+      </c>
+      <c r="L256" s="1" t="n">
+        <v>46127.45833333334</v>
+      </c>
+      <c r="M256" t="inlineStr">
+        <is>
+          <t>£200,000</t>
+        </is>
+      </c>
+      <c r="N256" s="1" t="n">
+        <v>46064</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Semiconductors and components for smart electronic platforms</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2403/overview/4b54c133-c9b2-4572-9cca-2a7a4f69e5b8</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>2026-02-20 10:32</t>
+        </is>
+      </c>
+      <c r="E257" s="1" t="n">
+        <v>46073.43888888889</v>
+      </c>
+      <c r="F257" t="b">
+        <v>1</v>
+      </c>
+      <c r="G257" t="inlineStr"/>
+      <c r="H257" t="b">
+        <v>0</v>
+      </c>
+      <c r="I257" t="inlineStr"/>
+      <c r="J257" t="inlineStr"/>
+      <c r="K257" t="inlineStr">
+        <is>
           <t>Wednesday 1 April 2026 11:00am</t>
         </is>
       </c>
-      <c r="L256" s="1" t="n">
+      <c r="L257" s="1" t="n">
         <v>46113.45833333334</v>
       </c>
-      <c r="M256" t="inlineStr">
+      <c r="M257" t="inlineStr">
         <is>
           <t>£2.0 million</t>
         </is>
       </c>
-      <c r="N256" s="1" t="n">
+      <c r="N257" s="1" t="n">
+        <v>46071</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Robotics Adoption Hubs</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2408/overview/ad7d7d36-af60-48be-91b0-f3208cf7c1d4</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>2026-02-24 10:43</t>
+        </is>
+      </c>
+      <c r="E258" s="1" t="n">
+        <v>46077.44652777778</v>
+      </c>
+      <c r="F258" t="b">
+        <v>1</v>
+      </c>
+      <c r="G258" t="inlineStr"/>
+      <c r="H258" t="b">
+        <v>0</v>
+      </c>
+      <c r="I258" t="inlineStr"/>
+      <c r="J258" t="inlineStr"/>
+      <c r="K258" t="inlineStr">
+        <is>
+          <t>Wednesday 15 April 2026 11:00am</t>
+        </is>
+      </c>
+      <c r="L258" s="1" t="n">
+        <v>46127.45833333334</v>
+      </c>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>£7.5 million</t>
+        </is>
+      </c>
+      <c r="N258" s="1" t="n">
+        <v>46071</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Innovate Funding Service</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Robotics Adoption Central Convening Body</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2409/overview/c7e5dd6a-9f34-4614-b548-214b76190c14</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>2026-02-24 10:43</t>
+        </is>
+      </c>
+      <c r="E259" s="1" t="n">
+        <v>46077.44652777778</v>
+      </c>
+      <c r="F259" t="b">
+        <v>1</v>
+      </c>
+      <c r="G259" t="inlineStr"/>
+      <c r="H259" t="b">
+        <v>0</v>
+      </c>
+      <c r="I259" t="inlineStr"/>
+      <c r="J259" t="inlineStr"/>
+      <c r="K259" t="inlineStr">
+        <is>
+          <t>Wednesday 15 April 2026 11:00am</t>
+        </is>
+      </c>
+      <c r="L259" s="1" t="n">
+        <v>46127.45833333334</v>
+      </c>
+      <c r="M259" t="inlineStr">
+        <is>
+          <t>£2.0 million</t>
+        </is>
+      </c>
+      <c r="N259" s="1" t="n">
         <v>46071</v>
       </c>
     </row>
@@ -15064,10 +15376,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C2" t="n">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3">
@@ -15077,10 +15389,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C3" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4">
@@ -15090,10 +15402,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="C4" t="n">
-        <v>255</v>
+        <v>258</v>
       </c>
     </row>
     <row r="5">

</xml_diff>